<commit_message>
MAJ absences 2026-06-09 16:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10514" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B7063E7-33FD-45F5-BE88-9D077F70A7F3}"/>
+  <xr:revisionPtr revIDLastSave="10520" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E56B82E-961F-4E3E-8B78-87A336BA54A0}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,115 +60,112 @@
     <t>MR PARKER</t>
   </si>
   <si>
-    <t>09/06</t>
+    <t>10/06</t>
   </si>
   <si>
     <t>*</t>
   </si>
   <si>
-    <t>MR HADJI</t>
-  </si>
-  <si>
-    <t>ONLY P1 TO P5</t>
-  </si>
-  <si>
-    <t>MR BAZIN</t>
-  </si>
-  <si>
-    <t>P1/S4L1-FRC</t>
+    <t>MRS HASSAINE</t>
+  </si>
+  <si>
+    <t>ONLY P3 TO P4</t>
+  </si>
+  <si>
+    <t>MR ANDERSEN</t>
+  </si>
+  <si>
+    <t>P3/S1L1-DAA</t>
+  </si>
+  <si>
+    <t>C104</t>
+  </si>
+  <si>
+    <t>MR NEKIC</t>
+  </si>
+  <si>
+    <t>P4/S3SCIDAA</t>
+  </si>
+  <si>
+    <t>D202</t>
+  </si>
+  <si>
+    <t>MRS GROBER</t>
+  </si>
+  <si>
+    <t>ONLY P3 TO P7</t>
+  </si>
+  <si>
+    <t>MR IONITA</t>
+  </si>
+  <si>
+    <t>P3/S2L3-FRA</t>
+  </si>
+  <si>
+    <t>D105</t>
+  </si>
+  <si>
+    <t>P5/S3L3-FRC</t>
+  </si>
+  <si>
+    <t>D106</t>
+  </si>
+  <si>
+    <t>MRS RIBA</t>
+  </si>
+  <si>
+    <t>P6/S1L2-FRA</t>
+  </si>
+  <si>
+    <t>Mrs PAVLIDOU</t>
+  </si>
+  <si>
+    <t>P7/S1L2-FRA</t>
+  </si>
+  <si>
+    <t>MRS WAECHTER</t>
+  </si>
+  <si>
+    <t>MR BERNET</t>
+  </si>
+  <si>
+    <t>P1/S6CHIFRB</t>
+  </si>
+  <si>
+    <t>D306</t>
+  </si>
+  <si>
+    <t>P2/S6CHIFRB</t>
+  </si>
+  <si>
+    <t>P3/S4PHYFRA</t>
+  </si>
+  <si>
+    <t>MRS COQUELIN</t>
+  </si>
+  <si>
+    <t>P5/S5CHIFRD</t>
+  </si>
+  <si>
+    <t>MRS LE GOALLER</t>
+  </si>
+  <si>
+    <t>ONLY P8 TO P9</t>
+  </si>
+  <si>
+    <t>MRS DEMARTINI</t>
+  </si>
+  <si>
+    <t>ONLY P1</t>
+  </si>
+  <si>
+    <t>Mrs RHEINHEIMER</t>
+  </si>
+  <si>
+    <t>P1/S1MATITB</t>
   </si>
   <si>
     <t>C210</t>
-  </si>
-  <si>
-    <t>P2/S4L1-FRB</t>
-  </si>
-  <si>
-    <t>C207</t>
-  </si>
-  <si>
-    <t>MRS XEROU</t>
-  </si>
-  <si>
-    <t>P4/S1L1-FRB</t>
-  </si>
-  <si>
-    <t>D103</t>
-  </si>
-  <si>
-    <t>MRS PINHEIRO</t>
-  </si>
-  <si>
-    <t>P5/S1L1-FRB</t>
-  </si>
-  <si>
-    <t>MRS MARTINEAU</t>
-  </si>
-  <si>
-    <t>MRS NOBIS</t>
-  </si>
-  <si>
-    <t>MRS RAYMONDAUD</t>
-  </si>
-  <si>
-    <t>MRS GROBER</t>
-  </si>
-  <si>
-    <t>P1/S4L1-FRA</t>
-  </si>
-  <si>
-    <t>D104</t>
-  </si>
-  <si>
-    <t>MRS DESROSIERS</t>
-  </si>
-  <si>
-    <t>P2/S4L1-FRA</t>
-  </si>
-  <si>
-    <t>MRS PIERSON</t>
-  </si>
-  <si>
-    <t>P4/S2L1-FRC</t>
-  </si>
-  <si>
-    <t>MRS SCHALLHORN</t>
-  </si>
-  <si>
-    <t>P5/S2L1-FRC</t>
-  </si>
-  <si>
-    <t>MR GILLIG</t>
-  </si>
-  <si>
-    <t>MR LESOURD</t>
-  </si>
-  <si>
-    <t>P3/S1SCHFRD</t>
-  </si>
-  <si>
-    <t>B007</t>
-  </si>
-  <si>
-    <t>MRS RODRIGUEZ</t>
-  </si>
-  <si>
-    <t>P4/S1SCHFRD</t>
-  </si>
-  <si>
-    <t>MRS COQUELIN</t>
-  </si>
-  <si>
-    <t>ONLY P4</t>
-  </si>
-  <si>
-    <t>MRS GALEZIOK</t>
-  </si>
-  <si>
-    <t>P4/S2SCIFRA</t>
-  </si>
-  <si>
-    <t>D208</t>
   </si>
 </sst>
 </file>
@@ -209,12 +206,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -294,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -324,6 +327,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -649,7 +655,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -719,95 +725,99 @@
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="10" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="C5" s="10" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="10" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
       <c r="C7" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+        <v>23</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>25</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
@@ -817,85 +827,68 @@
         <v>28</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="10"/>
+      <c r="A13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>33</v>
+        <v>38</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>39</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
-      <c r="C15" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>35</v>
-      </c>
+      <c r="C15" s="10"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -920,15 +913,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1226,14 +1210,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-10 08:40
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10520" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9E56B82E-961F-4E3E-8B78-87A336BA54A0}"/>
+  <xr:revisionPtr revIDLastSave="10538" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{765CDDE3-E0BB-4497-B393-668049BAF446}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
   <si>
     <t>NOMS</t>
   </si>
@@ -166,6 +166,33 @@
   </si>
   <si>
     <t>C210</t>
+  </si>
+  <si>
+    <t>Mrs KASTANIDOU</t>
+  </si>
+  <si>
+    <t>10/6</t>
+  </si>
+  <si>
+    <t>Mr. KLUPPELHOLZ</t>
+  </si>
+  <si>
+    <t>P3/S1SCH-ELA</t>
+  </si>
+  <si>
+    <t>B113</t>
+  </si>
+  <si>
+    <t>Mrs HERRIG</t>
+  </si>
+  <si>
+    <t>P5/S2SCH-ELA</t>
+  </si>
+  <si>
+    <t>Mrs FERRARI</t>
+  </si>
+  <si>
+    <t>ONLY P1 TO P5</t>
   </si>
 </sst>
 </file>
@@ -655,7 +682,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -877,18 +904,75 @@
       </c>
     </row>
     <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="A15" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="C16" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="1:5" ht="18">
+      <c r="A19" s="3"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+    </row>
+    <row r="20" spans="1:5" ht="18">
+      <c r="A20" s="3"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+    </row>
+    <row r="21" spans="1:5" ht="18">
+      <c r="A21" s="3"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -913,6 +997,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1210,23 +1303,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-10 08:45
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10538" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{765CDDE3-E0BB-4497-B393-668049BAF446}"/>
+  <xr:revisionPtr revIDLastSave="10544" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B28DB6F1-0C1D-44E2-B421-274A5EED6991}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="55">
   <si>
     <t>NOMS</t>
   </si>
@@ -193,6 +193,18 @@
   </si>
   <si>
     <t>ONLY P1 TO P5</t>
+  </si>
+  <si>
+    <t>Mr KUPPER</t>
+  </si>
+  <si>
+    <t>Mr PRIESS</t>
+  </si>
+  <si>
+    <t>P4/S2L1DEA</t>
+  </si>
+  <si>
+    <t>C111</t>
   </si>
 </sst>
 </file>
@@ -947,11 +959,21 @@
       <c r="E17" s="5"/>
     </row>
     <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="A18" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="19" spans="1:5" ht="18">
       <c r="A19" s="3"/>
@@ -982,30 +1004,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1303,8 +1301,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1312,5 +1334,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-10 08:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10544" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B28DB6F1-0C1D-44E2-B421-274A5EED6991}"/>
+  <xr:revisionPtr revIDLastSave="10550" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB44C422-6ECC-44D5-98FE-9C52951F0073}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="59">
   <si>
     <t>NOMS</t>
   </si>
@@ -198,13 +198,25 @@
     <t>Mr KUPPER</t>
   </si>
   <si>
-    <t>Mr PRIESS</t>
+    <t>Mrs GARCIA MARTIN</t>
   </si>
   <si>
     <t>P4/S2L1DEA</t>
   </si>
   <si>
     <t>C111</t>
+  </si>
+  <si>
+    <t>Mrs MENGES</t>
+  </si>
+  <si>
+    <t>Mrs PRIESS</t>
+  </si>
+  <si>
+    <t>P7/S5BIOFRB</t>
+  </si>
+  <si>
+    <t>D216</t>
   </si>
 </sst>
 </file>
@@ -983,11 +995,21 @@
       <c r="E19" s="5"/>
     </row>
     <row r="20" spans="1:5" ht="18">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
+      <c r="A20" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="21" spans="1:5" ht="18">
       <c r="A21" s="3"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 09:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10550" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB44C422-6ECC-44D5-98FE-9C52951F0073}"/>
+  <xr:revisionPtr revIDLastSave="10556" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25771D15-2859-4051-B5FF-89795C84DE8A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="61">
   <si>
     <t>NOMS</t>
   </si>
@@ -217,6 +217,12 @@
   </si>
   <si>
     <t>D216</t>
+  </si>
+  <si>
+    <t>Mrs BELPAUME</t>
+  </si>
+  <si>
+    <t>P8/S5L3DEA</t>
   </si>
 </sst>
 </file>
@@ -706,7 +712,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U22"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -1012,11 +1018,28 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
+      <c r="A21" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18">
+      <c r="A22" s="3"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 09:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10556" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25771D15-2859-4051-B5FF-89795C84DE8A}"/>
+  <xr:revisionPtr revIDLastSave="10561" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08AD9064-9A27-4BDF-B621-C961C2A92862}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
   <si>
     <t>NOMS</t>
   </si>
@@ -219,10 +219,7 @@
     <t>D216</t>
   </si>
   <si>
-    <t>Mrs BELPAUME</t>
-  </si>
-  <si>
-    <t>P8/S5L3DEA</t>
+    <t>Mrs MORAWSKA</t>
   </si>
 </sst>
 </file>
@@ -712,7 +709,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U22"/>
+  <dimension ref="A1:U23"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -1025,21 +1022,28 @@
         <v>36</v>
       </c>
       <c r="C21" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+    </row>
+    <row r="22" spans="1:5" ht="18">
+      <c r="A22" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="18">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="11"/>
+      <c r="B22" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="10"/>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
+    </row>
+    <row r="23" spans="1:5" ht="18">
+      <c r="A23" s="3"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 09:10
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10561" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08AD9064-9A27-4BDF-B621-C961C2A92862}"/>
+  <xr:revisionPtr revIDLastSave="10570" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61E614BC-EFCA-413C-BE0C-FBA389485FC9}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="63">
   <si>
     <t>NOMS</t>
   </si>
@@ -220,6 +220,15 @@
   </si>
   <si>
     <t>Mrs MORAWSKA</t>
+  </si>
+  <si>
+    <t>Mr SCHETTINO</t>
+  </si>
+  <si>
+    <t>P4/S1L3DEB</t>
+  </si>
+  <si>
+    <t>C112</t>
   </si>
 </sst>
 </file>
@@ -351,7 +360,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -384,6 +393,15 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -709,7 +727,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U23"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -1034,16 +1052,52 @@
       <c r="B22" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="10"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
+      <c r="C22" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="23" spans="1:5" ht="18">
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
-      <c r="C23" s="11"/>
+      <c r="C23" s="10" t="s">
+        <v>56</v>
+      </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
+    </row>
+    <row r="24" spans="1:5" ht="18">
+      <c r="A24" s="3"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+    </row>
+    <row r="25" spans="1:5" ht="18">
+      <c r="A25" s="3"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+    </row>
+    <row r="26" spans="1:5" ht="18">
+      <c r="A26" s="12"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+    </row>
+    <row r="27" spans="1:5" ht="18">
+      <c r="A27" s="12"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 09:15
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10570" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61E614BC-EFCA-413C-BE0C-FBA389485FC9}"/>
+  <xr:revisionPtr revIDLastSave="10572" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B24F0152-8AE8-4310-B5D9-BBC3F20402BB}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
   <si>
     <t>NOMS</t>
   </si>
@@ -229,6 +229,9 @@
   </si>
   <si>
     <t>C112</t>
+  </si>
+  <si>
+    <t>P5/S3L3DEC</t>
   </si>
 </sst>
 </file>
@@ -1068,8 +1071,12 @@
       <c r="C23" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
+      <c r="D23" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="24" spans="1:5" ht="18">
       <c r="A24" s="3"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 09:20
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10572" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B24F0152-8AE8-4310-B5D9-BBC3F20402BB}"/>
+  <xr:revisionPtr revIDLastSave="10573" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{553E67CF-5B3A-438F-AF60-896CF94F337A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
   <si>
     <t>NOMS</t>
   </si>
@@ -229,6 +229,9 @@
   </si>
   <si>
     <t>C112</t>
+  </si>
+  <si>
+    <t>Mrs KNIHAROVA</t>
   </si>
   <si>
     <t>P5/S3L3DEC</t>
@@ -1069,10 +1072,10 @@
       <c r="A23" s="3"/>
       <c r="B23" s="4"/>
       <c r="C23" s="10" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 09:35
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10573" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{553E67CF-5B3A-438F-AF60-896CF94F337A}"/>
+  <xr:revisionPtr revIDLastSave="10581" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC18A4DF-7547-45B1-A6F4-95D9BB05A559}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="66">
   <si>
     <t>NOMS</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>P5/S3L3DEC</t>
+  </si>
+  <si>
+    <t>Mr GILLIG</t>
   </si>
 </sst>
 </file>
@@ -733,7 +736,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -1082,25 +1085,31 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="18">
-      <c r="A24" s="3"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="10"/>
+      <c r="A24" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
     </row>
     <row r="25" spans="1:5" ht="18">
       <c r="A25" s="3"/>
       <c r="B25" s="4"/>
-      <c r="C25" s="11"/>
+      <c r="C25" s="10"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:5" ht="18">
-      <c r="A26" s="12"/>
-      <c r="B26" s="13"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
+      <c r="A26" s="3"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
     </row>
     <row r="27" spans="1:5" ht="18">
       <c r="A27" s="12"/>
@@ -1108,6 +1117,13 @@
       <c r="C27" s="14"/>
       <c r="D27" s="12"/>
       <c r="E27" s="12"/>
+    </row>
+    <row r="28" spans="1:5" ht="18">
+      <c r="A28" s="12"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 10:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30128"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10581" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC18A4DF-7547-45B1-A6F4-95D9BB05A559}"/>
+  <xr:revisionPtr revIDLastSave="10585" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{272F0E63-226E-4C09-BFB9-18C59FF68E05}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="68">
   <si>
     <t>NOMS</t>
   </si>
@@ -238,6 +238,12 @@
   </si>
   <si>
     <t>Mr GILLIG</t>
+  </si>
+  <si>
+    <t>Mr FRANKENREITER</t>
+  </si>
+  <si>
+    <t>ONLY P9</t>
   </si>
 </sst>
 </file>
@@ -404,13 +410,13 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -736,7 +742,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:U29"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -1098,25 +1104,31 @@
       <c r="E24" s="5"/>
     </row>
     <row r="25" spans="1:5" ht="18">
-      <c r="A25" s="3"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="10"/>
+      <c r="A25" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:5" ht="18">
       <c r="A26" s="3"/>
       <c r="B26" s="4"/>
-      <c r="C26" s="11"/>
+      <c r="C26" s="10"/>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
     </row>
     <row r="27" spans="1:5" ht="18">
-      <c r="A27" s="12"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
+      <c r="A27" s="3"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
     </row>
     <row r="28" spans="1:5" ht="18">
       <c r="A28" s="12"/>
@@ -1124,6 +1136,13 @@
       <c r="C28" s="14"/>
       <c r="D28" s="12"/>
       <c r="E28" s="12"/>
+    </row>
+    <row r="29" spans="1:5" ht="18">
+      <c r="A29" s="12"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1133,6 +1152,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1430,15 +1458,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1455,11 +1474,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-10 16:20
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10585" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{272F0E63-226E-4C09-BFB9-18C59FF68E05}"/>
+  <xr:revisionPtr revIDLastSave="10588" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEF4023A-4101-4932-99F9-F1C37B070C2C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,193 +57,49 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MR PARKER</t>
-  </si>
-  <si>
-    <t>10/06</t>
+    <t>MRS LE GOALLER</t>
+  </si>
+  <si>
+    <t>ONLY P8 TO P9</t>
   </si>
   <si>
     <t>*</t>
   </si>
   <si>
-    <t>MRS HASSAINE</t>
-  </si>
-  <si>
-    <t>ONLY P3 TO P4</t>
-  </si>
-  <si>
-    <t>MR ANDERSEN</t>
-  </si>
-  <si>
-    <t>P3/S1L1-DAA</t>
-  </si>
-  <si>
-    <t>C104</t>
-  </si>
-  <si>
-    <t>MR NEKIC</t>
-  </si>
-  <si>
-    <t>P4/S3SCIDAA</t>
-  </si>
-  <si>
-    <t>D202</t>
-  </si>
-  <si>
-    <t>MRS GROBER</t>
-  </si>
-  <si>
-    <t>ONLY P3 TO P7</t>
-  </si>
-  <si>
-    <t>MR IONITA</t>
-  </si>
-  <si>
-    <t>P3/S2L3-FRA</t>
-  </si>
-  <si>
-    <t>D105</t>
-  </si>
-  <si>
-    <t>P5/S3L3-FRC</t>
-  </si>
-  <si>
-    <t>D106</t>
-  </si>
-  <si>
-    <t>MRS RIBA</t>
-  </si>
-  <si>
-    <t>P6/S1L2-FRA</t>
-  </si>
-  <si>
-    <t>Mrs PAVLIDOU</t>
-  </si>
-  <si>
-    <t>P7/S1L2-FRA</t>
-  </si>
-  <si>
-    <t>MRS WAECHTER</t>
-  </si>
-  <si>
-    <t>MR BERNET</t>
-  </si>
-  <si>
-    <t>P1/S6CHIFRB</t>
-  </si>
-  <si>
-    <t>D306</t>
-  </si>
-  <si>
-    <t>P2/S6CHIFRB</t>
-  </si>
-  <si>
-    <t>P3/S4PHYFRA</t>
-  </si>
-  <si>
-    <t>MRS COQUELIN</t>
-  </si>
-  <si>
-    <t>P5/S5CHIFRD</t>
-  </si>
-  <si>
-    <t>MRS LE GOALLER</t>
-  </si>
-  <si>
-    <t>ONLY P8 TO P9</t>
-  </si>
-  <si>
-    <t>MRS DEMARTINI</t>
-  </si>
-  <si>
-    <t>ONLY P1</t>
-  </si>
-  <si>
-    <t>Mrs RHEINHEIMER</t>
-  </si>
-  <si>
-    <t>P1/S1MATITB</t>
-  </si>
-  <si>
-    <t>C210</t>
-  </si>
-  <si>
-    <t>Mrs KASTANIDOU</t>
-  </si>
-  <si>
-    <t>10/6</t>
-  </si>
-  <si>
-    <t>Mr. KLUPPELHOLZ</t>
-  </si>
-  <si>
-    <t>P3/S1SCH-ELA</t>
-  </si>
-  <si>
-    <t>B113</t>
-  </si>
-  <si>
-    <t>Mrs HERRIG</t>
-  </si>
-  <si>
-    <t>P5/S2SCH-ELA</t>
-  </si>
-  <si>
-    <t>Mrs FERRARI</t>
-  </si>
-  <si>
-    <t>ONLY P1 TO P5</t>
-  </si>
-  <si>
-    <t>Mr KUPPER</t>
-  </si>
-  <si>
-    <t>Mrs GARCIA MARTIN</t>
-  </si>
-  <si>
-    <t>P4/S2L1DEA</t>
-  </si>
-  <si>
-    <t>C111</t>
-  </si>
-  <si>
-    <t>Mrs MENGES</t>
-  </si>
-  <si>
-    <t>Mrs PRIESS</t>
-  </si>
-  <si>
-    <t>P7/S5BIOFRB</t>
-  </si>
-  <si>
-    <t>D216</t>
-  </si>
-  <si>
-    <t>Mrs MORAWSKA</t>
-  </si>
-  <si>
-    <t>Mr SCHETTINO</t>
-  </si>
-  <si>
-    <t>P4/S1L3DEB</t>
-  </si>
-  <si>
-    <t>C112</t>
-  </si>
-  <si>
-    <t>Mrs KNIHAROVA</t>
-  </si>
-  <si>
-    <t>P5/S3L3DEC</t>
-  </si>
-  <si>
-    <t>Mr GILLIG</t>
-  </si>
-  <si>
-    <t>Mr FRANKENREITER</t>
-  </si>
-  <si>
-    <t>ONLY P9</t>
+    <t>Mrs GIORGERINI</t>
+  </si>
+  <si>
+    <t>ONLY P7 TO P9</t>
+  </si>
+  <si>
+    <t>Mr BENREKIA</t>
+  </si>
+  <si>
+    <t>Mrs ZAJICKOVA</t>
+  </si>
+  <si>
+    <t>11/6</t>
+  </si>
+  <si>
+    <t>Work has been assigned</t>
+  </si>
+  <si>
+    <t>P1/S5L1-CSA</t>
+  </si>
+  <si>
+    <t>P2/S4L1-CSA</t>
+  </si>
+  <si>
+    <t>Go to Library</t>
+  </si>
+  <si>
+    <t>P3/S2L1-CSA</t>
+  </si>
+  <si>
+    <t>Library</t>
+  </si>
+  <si>
+    <t>P4/S3L1-CSA</t>
   </si>
 </sst>
 </file>
@@ -375,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -405,9 +261,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -742,7 +595,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U29"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -799,43 +652,35 @@
         <v>9</v>
       </c>
       <c r="C3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" ht="18">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="18">
-      <c r="A4" s="3"/>
       <c r="B4" s="4"/>
-      <c r="C4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>15</v>
-      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
@@ -845,304 +690,65 @@
         <v>13</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
       <c r="C7" s="10" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="10" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
-      <c r="C10" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="C10" s="10"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="A11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" spans="1:5" ht="18">
-      <c r="A20" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-    </row>
-    <row r="22" spans="1:5" ht="18">
-      <c r="A22" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="18">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="18">
-      <c r="A24" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5" ht="18">
-      <c r="A25" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-    </row>
-    <row r="26" spans="1:5" ht="18">
-      <c r="A26" s="3"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-    </row>
-    <row r="27" spans="1:5" ht="18">
-      <c r="A27" s="3"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="11"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-    </row>
-    <row r="28" spans="1:5" ht="18">
-      <c r="A28" s="12"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-    </row>
-    <row r="29" spans="1:5" ht="18">
-      <c r="A29" s="12"/>
-      <c r="B29" s="13"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1152,6 +758,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1160,7 +781,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1458,29 +1079,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-11 08:45
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10588" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEF4023A-4101-4932-99F9-F1C37B070C2C}"/>
+  <xr:revisionPtr revIDLastSave="10608" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76FD52BE-2147-43E1-BC75-8BEEBB38B7C0}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
   <si>
     <t>NOMS</t>
   </si>
@@ -100,6 +100,30 @@
   </si>
   <si>
     <t>P4/S3L1-CSA</t>
+  </si>
+  <si>
+    <t>Mrs ZARB HABER</t>
+  </si>
+  <si>
+    <t>en attente de remplacement</t>
+  </si>
+  <si>
+    <t>Mrs VORNICESCU</t>
+  </si>
+  <si>
+    <t>M KARAGIANNIDIS</t>
+  </si>
+  <si>
+    <t>ONLY P9</t>
+  </si>
+  <si>
+    <t>Mrs GESTHUISEN</t>
+  </si>
+  <si>
+    <t>Mrs CHLUMSKA</t>
+  </si>
+  <si>
+    <t>ONLY P8</t>
   </si>
 </sst>
 </file>
@@ -595,7 +619,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -722,33 +746,84 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="10"/>
+    <row r="9" spans="1:12" ht="36">
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>21</v>
+      </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="10"/>
+    <row r="10" spans="1:12" ht="36">
+      <c r="A10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>21</v>
+      </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
+    <row r="11" spans="1:12" ht="36">
+      <c r="A11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="36">
+      <c r="A12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="36">
+      <c r="A13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="11"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -758,30 +833,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1079,8 +1130,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1088,5 +1163,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-11 08:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10608" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76FD52BE-2147-43E1-BC75-8BEEBB38B7C0}"/>
+  <xr:revisionPtr revIDLastSave="10620" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6D20E7F-5762-4382-BDF2-7B8825918E65}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
   <si>
     <t>NOMS</t>
   </si>
@@ -111,6 +111,15 @@
     <t>Mrs VORNICESCU</t>
   </si>
   <si>
+    <t>Mrs GRIRA</t>
+  </si>
+  <si>
+    <t>P5/S4PHY-DEB</t>
+  </si>
+  <si>
+    <t>D310</t>
+  </si>
+  <si>
     <t>M KARAGIANNIDIS</t>
   </si>
   <si>
@@ -118,6 +127,21 @@
   </si>
   <si>
     <t>Mrs GESTHUISEN</t>
+  </si>
+  <si>
+    <t>Mrs DESROSIERS</t>
+  </si>
+  <si>
+    <t>P3/MOR-DEA</t>
+  </si>
+  <si>
+    <t>C110</t>
+  </si>
+  <si>
+    <t>Mrs SADELER</t>
+  </si>
+  <si>
+    <t>P8/S2L3-DEC</t>
   </si>
   <si>
     <t>Mrs CHLUMSKA</t>
@@ -619,7 +643,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -759,7 +783,7 @@
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:12" ht="36">
+    <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
@@ -767,56 +791,70 @@
         <v>12</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" ht="36">
+        <v>23</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" spans="1:12" ht="36">
+    <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="36">
+      <c r="A14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" ht="36">
-      <c r="A13" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="11"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="11"/>
@@ -824,6 +862,13 @@
       <c r="C15" s="13"/>
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-11 08:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10620" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6D20E7F-5762-4382-BDF2-7B8825918E65}"/>
+  <xr:revisionPtr revIDLastSave="10634" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC626603-3487-478E-8A09-58EBF4C722BB}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
   <si>
     <t>NOMS</t>
   </si>
@@ -105,7 +105,19 @@
     <t>Mrs ZARB HABER</t>
   </si>
   <si>
-    <t>en attente de remplacement</t>
+    <t>Mrs TOURA</t>
+  </si>
+  <si>
+    <t>P3/S1L2-END</t>
+  </si>
+  <si>
+    <t>C002</t>
+  </si>
+  <si>
+    <t>Mrs DI SALVATORE</t>
+  </si>
+  <si>
+    <t>P4/S1L2-END</t>
   </si>
   <si>
     <t>Mrs VORNICESCU</t>
@@ -148,6 +160,15 @@
   </si>
   <si>
     <t>ONLY P8</t>
+  </si>
+  <si>
+    <t>M. ROLL</t>
+  </si>
+  <si>
+    <t>P8/S2L3-ENB</t>
+  </si>
+  <si>
+    <t>B102</t>
   </si>
 </sst>
 </file>
@@ -643,7 +664,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -770,7 +791,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="36">
+    <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -780,24 +801,24 @@
       <c r="C9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="D9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
       <c r="C10" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
@@ -805,70 +826,105 @@
         <v>26</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
       <c r="C13" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="36">
-      <c r="A14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="4" t="s">
         <v>35</v>
       </c>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
       <c r="C14" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+        <v>36</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="11"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
+      <c r="A15" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="11"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+    </row>
+    <row r="19" spans="1:5" ht="18">
+      <c r="A19" s="11"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-11 09:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10634" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CC626603-3487-478E-8A09-58EBF4C722BB}"/>
+  <xr:revisionPtr revIDLastSave="10644" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8F1A08B-895F-4B1D-9874-81F1B4A6D68F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="49">
   <si>
     <t>NOMS</t>
   </si>
@@ -169,6 +169,24 @@
   </si>
   <si>
     <t>B102</t>
+  </si>
+  <si>
+    <t>Mrs FAZZARI</t>
+  </si>
+  <si>
+    <t>Mrs DEMARTINI</t>
+  </si>
+  <si>
+    <t>P2/S1SCH-ITA</t>
+  </si>
+  <si>
+    <t>C206</t>
+  </si>
+  <si>
+    <t>Mrs ARGYRI</t>
+  </si>
+  <si>
+    <t>P7/SCH-ITB</t>
   </si>
 </sst>
 </file>
@@ -899,17 +917,31 @@
       </c>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="A16" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="18">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="5"/>
+      <c r="C17" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="E17" s="5"/>
     </row>
     <row r="18" spans="1:5" ht="18">
@@ -934,6 +966,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1231,32 +1287,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1264,5 +1296,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-11 09:10
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10644" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8F1A08B-895F-4B1D-9874-81F1B4A6D68F}"/>
+  <xr:revisionPtr revIDLastSave="10648" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4A18B83-23C4-4436-B95E-F30C9374F65B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
   <si>
     <t>NOMS</t>
   </si>
@@ -186,7 +186,7 @@
     <t>Mrs ARGYRI</t>
   </si>
   <si>
-    <t>P7/SCH-ITB</t>
+    <t>P7/S2SCH-ITB</t>
   </si>
 </sst>
 </file>
@@ -318,7 +318,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -357,6 +357,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -682,7 +691,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U19"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -917,46 +926,62 @@
       </c>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B17" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C17" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="10" t="s">
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="11"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
+      <c r="E18" s="5" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="11"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+    </row>
+    <row r="20" spans="1:5" ht="18">
+      <c r="A20" s="11"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+    </row>
+    <row r="21" spans="1:5" ht="18">
+      <c r="A21" s="11"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-11 09:40
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10648" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4A18B83-23C4-4436-B95E-F30C9374F65B}"/>
+  <xr:revisionPtr revIDLastSave="10649" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D596876-5598-4A36-AFE8-3ED92B32456F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="47">
   <si>
     <t>NOMS</t>
   </si>
@@ -130,12 +130,6 @@
   </si>
   <si>
     <t>D310</t>
-  </si>
-  <si>
-    <t>M KARAGIANNIDIS</t>
-  </si>
-  <si>
-    <t>ONLY P9</t>
   </si>
   <si>
     <t>Mrs GESTHUISEN</t>
@@ -691,7 +685,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -870,104 +864,98 @@
         <v>30</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="D12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E15" s="5" t="s">
+      <c r="C16" s="10" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="D16" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>12</v>
-      </c>
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
       <c r="C17" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>46</v>
-      </c>
     </row>
     <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>46</v>
-      </c>
+      <c r="A18" s="14"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
     </row>
     <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="14"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" ht="18">
       <c r="A20" s="11"/>
@@ -975,13 +963,6 @@
       <c r="C20" s="13"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
-    </row>
-    <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-11 11:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10649" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D596876-5598-4A36-AFE8-3ED92B32456F}"/>
+  <xr:revisionPtr revIDLastSave="10653" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50637A2F-969C-44E9-AADF-4315D2A79BB8}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
   <si>
     <t>NOMS</t>
   </si>
@@ -163,6 +163,12 @@
   </si>
   <si>
     <t>B102</t>
+  </si>
+  <si>
+    <t>Mrs BRODARIC</t>
+  </si>
+  <si>
+    <t>ONLY P3</t>
   </si>
   <si>
     <t>Mrs FAZZARI</t>
@@ -907,40 +913,46 @@
       </c>
     </row>
     <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="10"/>
+      <c r="A15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>7</v>
+      </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>12</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D17" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>46</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18">

</xml_diff>

<commit_message>
MAJ absences 2026-06-11 16:15
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10653" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{50637A2F-969C-44E9-AADF-4315D2A79BB8}"/>
+  <xr:revisionPtr revIDLastSave="10655" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C07FD44-D8DB-44F2-AA02-B4A7EEA3B8C0}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,136 +57,118 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MRS LE GOALLER</t>
-  </si>
-  <si>
-    <t>ONLY P8 TO P9</t>
+    <t>Mrs KNIHAROVA</t>
+  </si>
+  <si>
+    <t>12/6</t>
+  </si>
+  <si>
+    <t>Go to the library</t>
+  </si>
+  <si>
+    <t>P4/S3L1-SKA</t>
+  </si>
+  <si>
+    <t>Go to the libray</t>
+  </si>
+  <si>
+    <t>Mrs ZAJICKOVA</t>
+  </si>
+  <si>
+    <t>ONLY  P2 + P8</t>
+  </si>
+  <si>
+    <t>en attente de remplacement</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>P8</t>
+  </si>
+  <si>
+    <t>Mrs PINHEIRO</t>
+  </si>
+  <si>
+    <t>ONLY P6 TO P9</t>
   </si>
   <si>
     <t>*</t>
   </si>
   <si>
-    <t>Mrs GIORGERINI</t>
-  </si>
-  <si>
-    <t>ONLY P7 TO P9</t>
-  </si>
-  <si>
-    <t>Mr BENREKIA</t>
-  </si>
-  <si>
-    <t>Mrs ZAJICKOVA</t>
-  </si>
-  <si>
-    <t>11/6</t>
-  </si>
-  <si>
-    <t>Work has been assigned</t>
-  </si>
-  <si>
-    <t>P1/S5L1-CSA</t>
-  </si>
-  <si>
-    <t>P2/S4L1-CSA</t>
-  </si>
-  <si>
-    <t>Go to Library</t>
-  </si>
-  <si>
-    <t>P3/S2L1-CSA</t>
-  </si>
-  <si>
-    <t>Library</t>
-  </si>
-  <si>
-    <t>P4/S3L1-CSA</t>
+    <t>M LEDUC</t>
+  </si>
+  <si>
+    <t>M ROLL</t>
+  </si>
+  <si>
+    <t>ONLY P5 TO P9</t>
+  </si>
+  <si>
+    <t>M IONITA</t>
   </si>
   <si>
     <t>Mrs ZARB HABER</t>
   </si>
   <si>
-    <t>Mrs TOURA</t>
-  </si>
-  <si>
-    <t>P3/S1L2-END</t>
-  </si>
-  <si>
-    <t>C002</t>
+    <t>ONLY P9</t>
+  </si>
+  <si>
+    <t>Mrs ORMASTI</t>
+  </si>
+  <si>
+    <t>M. GILLIG</t>
+  </si>
+  <si>
+    <t>P1/S1SCH-FRA</t>
+  </si>
+  <si>
+    <t>A001</t>
+  </si>
+  <si>
+    <t>M. SNAPPE</t>
+  </si>
+  <si>
+    <t>P2/S1SCH-FRA</t>
+  </si>
+  <si>
+    <t>P7/S1SCH-FRB</t>
+  </si>
+  <si>
+    <t>Mrs FORET-TOUSSAINT</t>
+  </si>
+  <si>
+    <t>ONLY P3</t>
+  </si>
+  <si>
+    <t>Mr BERRICHI</t>
+  </si>
+  <si>
+    <t>P3/S2MOR-FRC</t>
+  </si>
+  <si>
+    <t>B206</t>
   </si>
   <si>
     <t>Mrs DI SALVATORE</t>
   </si>
   <si>
-    <t>P4/S1L2-END</t>
-  </si>
-  <si>
-    <t>Mrs VORNICESCU</t>
-  </si>
-  <si>
-    <t>Mrs GRIRA</t>
-  </si>
-  <si>
-    <t>P5/S4PHY-DEB</t>
-  </si>
-  <si>
-    <t>D310</t>
-  </si>
-  <si>
-    <t>Mrs GESTHUISEN</t>
-  </si>
-  <si>
-    <t>Mrs DESROSIERS</t>
-  </si>
-  <si>
-    <t>P3/MOR-DEA</t>
-  </si>
-  <si>
-    <t>C110</t>
-  </si>
-  <si>
-    <t>Mrs SADELER</t>
-  </si>
-  <si>
-    <t>P8/S2L3-DEC</t>
-  </si>
-  <si>
-    <t>Mrs CHLUMSKA</t>
-  </si>
-  <si>
-    <t>ONLY P8</t>
-  </si>
-  <si>
-    <t>M. ROLL</t>
-  </si>
-  <si>
-    <t>P8/S2L3-ENB</t>
-  </si>
-  <si>
-    <t>B102</t>
-  </si>
-  <si>
-    <t>Mrs BRODARIC</t>
-  </si>
-  <si>
-    <t>ONLY P3</t>
-  </si>
-  <si>
-    <t>Mrs FAZZARI</t>
-  </si>
-  <si>
-    <t>Mrs DEMARTINI</t>
-  </si>
-  <si>
-    <t>P2/S1SCH-ITA</t>
+    <t>Mrs GALEZIOK</t>
+  </si>
+  <si>
+    <t>P3/S2RCA-FRA</t>
+  </si>
+  <si>
+    <t>A003</t>
+  </si>
+  <si>
+    <t>Mrs ARGYRI</t>
+  </si>
+  <si>
+    <t>P7/S2SCH-ITB</t>
   </si>
   <si>
     <t>C206</t>
-  </si>
-  <si>
-    <t>Mrs ARGYRI</t>
-  </si>
-  <si>
-    <t>P7/S2SCH-ITB</t>
   </si>
 </sst>
 </file>
@@ -318,7 +300,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -359,13 +341,10 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -691,7 +670,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -737,162 +716,162 @@
       <c r="C2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:12" ht="18">
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="36">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="5"/>
+        <v>12</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:12" ht="18">
-      <c r="A4" s="3" t="s">
-        <v>10</v>
-      </c>
+    <row r="4" spans="1:12" ht="36">
+      <c r="A4" s="3"/>
       <c r="B4" s="4"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="5"/>
+      <c r="C4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>14</v>
+      </c>
       <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>7</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
+      <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>16</v>
+      </c>
       <c r="C6" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>7</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
+      <c r="A7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="C7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8" spans="1:12" ht="18">
+      <c r="A8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="C8" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="5" t="s">
         <v>23</v>
       </c>
+      <c r="C9" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="10" t="s">
+      <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
+      <c r="B10" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="D10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="10" t="s">
+      <c r="D12" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="10" t="s">
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="B13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="C13" s="10" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="10" t="s">
+      <c r="D13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
@@ -900,81 +879,51 @@
         <v>36</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="D14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="5" t="s">
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="10" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
+      <c r="D15" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>46</v>
-      </c>
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
     </row>
     <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>46</v>
-      </c>
+      <c r="A17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
     </row>
     <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="14"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-    </row>
-    <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="11"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-    </row>
-    <row r="20" spans="1:5" ht="18">
-      <c r="A20" s="11"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -984,6 +933,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -996,15 +954,6 @@
     <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1306,11 +1255,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-12 08:35
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10655" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C07FD44-D8DB-44F2-AA02-B4A7EEA3B8C0}"/>
+  <xr:revisionPtr revIDLastSave="10665" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00E658C5-3C55-4ECA-A70E-97BC916DA775}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
   <si>
     <t>NOMS</t>
   </si>
@@ -112,6 +112,12 @@
   </si>
   <si>
     <t>ONLY P9</t>
+  </si>
+  <si>
+    <t>Mrs GESTHUISEN</t>
+  </si>
+  <si>
+    <t>Mrs VORNICESCU</t>
   </si>
   <si>
     <t>Mrs ORMASTI</t>
@@ -670,7 +676,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -814,7 +820,7 @@
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:12" ht="18">
+    <row r="10" spans="1:12" ht="36">
       <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
@@ -822,108 +828,134 @@
         <v>6</v>
       </c>
       <c r="C10" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:12" ht="36">
+      <c r="A11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="B11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="15" t="s">
+      <c r="D12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="5" t="s">
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="15" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="E14" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="B15" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="C15" s="10" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
+      <c r="D15" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="10" t="s">
+      <c r="E15" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="5" t="s">
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="B16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="10" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="10" t="s">
+      <c r="D16" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="5" t="s">
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="10" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="11"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
+      <c r="D17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="18" spans="1:5" ht="18">
       <c r="A18" s="11"/>
       <c r="B18" s="12"/>
-      <c r="C18" s="13"/>
+      <c r="C18" s="14"/>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
+    </row>
+    <row r="19" spans="1:5" ht="18">
+      <c r="A19" s="11"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+    </row>
+    <row r="20" spans="1:5" ht="18">
+      <c r="A20" s="11"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -933,15 +965,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -954,6 +977,15 @@
     <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1255,11 +1287,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-12 08:40
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10665" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00E658C5-3C55-4ECA-A70E-97BC916DA775}"/>
+  <xr:revisionPtr revIDLastSave="10673" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2008B520-5112-4745-B94E-C1CABC95F80C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
   <si>
     <t>NOMS</t>
   </si>
@@ -118,6 +118,21 @@
   </si>
   <si>
     <t>Mrs VORNICESCU</t>
+  </si>
+  <si>
+    <t>M CHEILAS</t>
+  </si>
+  <si>
+    <t>ONLY P1</t>
+  </si>
+  <si>
+    <t>M ZAHARIA</t>
+  </si>
+  <si>
+    <t>P1/S1SCI-ENB</t>
+  </si>
+  <si>
+    <t>D204</t>
   </si>
   <si>
     <t>Mrs ORMASTI</t>
@@ -676,7 +691,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -851,59 +866,59 @@
         <v>26</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
       <c r="C13" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="15" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="D15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="18">
@@ -911,42 +926,52 @@
         <v>38</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C16" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
       <c r="C17" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="11"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="19" spans="1:5" ht="18">
       <c r="A19" s="11"/>
       <c r="B19" s="12"/>
-      <c r="C19" s="13"/>
+      <c r="C19" s="14"/>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
     </row>
@@ -956,6 +981,13 @@
       <c r="C20" s="13"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
+    </row>
+    <row r="21" spans="1:5" ht="18">
+      <c r="A21" s="11"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-12 08:45
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10673" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2008B520-5112-4745-B94E-C1CABC95F80C}"/>
+  <xr:revisionPtr revIDLastSave="10688" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A3635F5-337F-43B7-9C6F-104EE7BE29D4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="56">
   <si>
     <t>NOMS</t>
   </si>
@@ -118,6 +118,24 @@
   </si>
   <si>
     <t>Mrs VORNICESCU</t>
+  </si>
+  <si>
+    <t>Mrs MONTEIRO</t>
+  </si>
+  <si>
+    <t>P2/S4XMADEA</t>
+  </si>
+  <si>
+    <t>D312</t>
+  </si>
+  <si>
+    <t>M HENTSCHEL</t>
+  </si>
+  <si>
+    <t>P4/S5PHYDEA</t>
+  </si>
+  <si>
+    <t>P7/S2MATDEB</t>
   </si>
   <si>
     <t>M CHEILAS</t>
@@ -691,7 +709,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U21"/>
+  <dimension ref="A1:U25"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -848,146 +866,188 @@
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" spans="1:12" ht="36">
-      <c r="A11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>12</v>
-      </c>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="15"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="E12" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="5" t="s">
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="E13" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="15" t="s">
-        <v>35</v>
-      </c>
+      <c r="C14" s="15"/>
       <c r="D14" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>34</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
-      <c r="C15" s="15" t="s">
-        <v>32</v>
-      </c>
+      <c r="C15" s="15"/>
       <c r="D15" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>34</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>40</v>
+        <v>33</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>34</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18">
       <c r="A17" s="3" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="E17" s="5" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="18">
+      <c r="A19" s="3"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="18">
+      <c r="A20" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="5" t="s">
+    </row>
+    <row r="21" spans="1:5" ht="18">
+      <c r="A21" s="3" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="11"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-    </row>
-    <row r="20" spans="1:5" ht="18">
-      <c r="A20" s="11"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-    </row>
-    <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
+      <c r="B21" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18">
+      <c r="A22" s="3"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="18">
+      <c r="A23" s="11"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+    </row>
+    <row r="24" spans="1:5" ht="18">
+      <c r="A24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+    </row>
+    <row r="25" spans="1:5" ht="18">
+      <c r="A25" s="11"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-12 08:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10688" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A3635F5-337F-43B7-9C6F-104EE7BE29D4}"/>
+  <xr:revisionPtr revIDLastSave="10706" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0D6DCB3-F64C-4643-A828-0F8E10AF2AEC}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
   <si>
     <t>NOMS</t>
   </si>
@@ -117,6 +117,24 @@
     <t>Mrs GESTHUISEN</t>
   </si>
   <si>
+    <t>M. KLOPP</t>
+  </si>
+  <si>
+    <t>P4/S4L4-DEA</t>
+  </si>
+  <si>
+    <t>C110</t>
+  </si>
+  <si>
+    <t>Mrs CASTELLO</t>
+  </si>
+  <si>
+    <t>P5/S4L4-DEA</t>
+  </si>
+  <si>
+    <t>P8/S6L1-DEA</t>
+  </si>
+  <si>
     <t>Mrs VORNICESCU</t>
   </si>
   <si>
@@ -135,7 +153,16 @@
     <t>P4/S5PHYDEA</t>
   </si>
   <si>
+    <t>M. CHEILAS</t>
+  </si>
+  <si>
     <t>P7/S2MATDEB</t>
+  </si>
+  <si>
+    <t>MRS MYSIRLAKI</t>
+  </si>
+  <si>
+    <t>P8/S5MA6DEA</t>
   </si>
   <si>
     <t>M CHEILAS</t>
@@ -709,7 +736,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -853,7 +880,7 @@
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:12" ht="36">
+    <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
@@ -861,184 +888,208 @@
         <v>6</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+        <v>25</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="C11" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="D12" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
       <c r="C13" s="15" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="15"/>
+      <c r="C14" s="15" t="s">
+        <v>35</v>
+      </c>
       <c r="D14" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" s="5"/>
+        <v>36</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
-      <c r="C15" s="15"/>
+      <c r="C15" s="15" t="s">
+        <v>37</v>
+      </c>
       <c r="D15" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E15" s="5"/>
+        <v>38</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
       <c r="C16" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18">
       <c r="A17" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B17" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
       <c r="C18" s="15" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="18">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="15" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18">
-      <c r="A20" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>46</v>
+      <c r="A20" s="3"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="15" t="s">
+        <v>47</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="18">
       <c r="A21" s="3" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18">
-      <c r="A22" s="3"/>
-      <c r="B22" s="4"/>
+      <c r="A22" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="C22" s="10" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="18">
-      <c r="A23" s="11"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
+      <c r="A23" s="3"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="24" spans="1:5" ht="18">
       <c r="A24" s="11"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="13"/>
+      <c r="C24" s="14"/>
       <c r="D24" s="11"/>
       <c r="E24" s="11"/>
     </row>
@@ -1048,6 +1099,13 @@
       <c r="C25" s="13"/>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
+    </row>
+    <row r="26" spans="1:5" ht="18">
+      <c r="A26" s="11"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-12 08:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10706" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0D6DCB3-F64C-4643-A828-0F8E10AF2AEC}"/>
+  <xr:revisionPtr revIDLastSave="10719" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99827395-6856-4C0B-81F2-4D2C64AF301B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
   <si>
     <t>NOMS</t>
   </si>
@@ -114,6 +114,18 @@
     <t>ONLY P9</t>
   </si>
   <si>
+    <t>Mrs LE GOALLER</t>
+  </si>
+  <si>
+    <t>Mrs NECHITA</t>
+  </si>
+  <si>
+    <t>P5/S2L2-DEA</t>
+  </si>
+  <si>
+    <t>B217</t>
+  </si>
+  <si>
     <t>Mrs GESTHUISEN</t>
   </si>
   <si>
@@ -132,9 +144,6 @@
     <t>P5/S4L4-DEA</t>
   </si>
   <si>
-    <t>P8/S6L1-DEA</t>
-  </si>
-  <si>
     <t>Mrs VORNICESCU</t>
   </si>
   <si>
@@ -226,15 +235,6 @@
   </si>
   <si>
     <t>A003</t>
-  </si>
-  <si>
-    <t>Mrs ARGYRI</t>
-  </si>
-  <si>
-    <t>P7/S2SCH-ITB</t>
-  </si>
-  <si>
-    <t>C206</t>
   </si>
 </sst>
 </file>
@@ -736,7 +736,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U25"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -898,198 +898,196 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C11" s="15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="15" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
       <c r="C14" s="15" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>37</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="15" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18">
       <c r="A17" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18">
       <c r="A18" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="18">
       <c r="A19" s="3"/>
       <c r="B19" s="4"/>
       <c r="C19" s="15" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="15" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D20" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="18">
       <c r="A21" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18">
       <c r="A22" s="3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="18">
-      <c r="A23" s="3"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>64</v>
-      </c>
+      <c r="A23" s="11"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
     </row>
     <row r="24" spans="1:5" ht="18">
       <c r="A24" s="11"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="14"/>
+      <c r="C24" s="13"/>
       <c r="D24" s="11"/>
       <c r="E24" s="11"/>
     </row>
@@ -1099,13 +1097,6 @@
       <c r="C25" s="13"/>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
-    </row>
-    <row r="26" spans="1:5" ht="18">
-      <c r="A26" s="11"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1115,6 +1106,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -1127,15 +1127,6 @@
     <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1437,11 +1428,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-12 09:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10719" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99827395-6856-4C0B-81F2-4D2C64AF301B}"/>
+  <xr:revisionPtr revIDLastSave="10731" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DFDC0C7-389B-4555-AA6C-DDF9167C9741}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$3</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
     <definedName name="toShow">Feuil1!$A:$E</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,61 +60,97 @@
     <t>Mrs KNIHAROVA</t>
   </si>
   <si>
+    <t>12/6 ONLY P1 TO P6</t>
+  </si>
+  <si>
+    <t>Mrs THEODOROU</t>
+  </si>
+  <si>
+    <t>P4/S3L1-SKA</t>
+  </si>
+  <si>
+    <t>Go to the libray</t>
+  </si>
+  <si>
+    <t>Mrs JUHASZ</t>
+  </si>
+  <si>
+    <t>P6/S1L1-SKA</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Verdana"/>
+      </rPr>
+      <t>C10</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Verdana"/>
+      </rPr>
+      <t>6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Verdana"/>
+      </rPr>
+      <t xml:space="preserve">   attention!</t>
+    </r>
+  </si>
+  <si>
+    <t>Mrs ZAJICKOVA</t>
+  </si>
+  <si>
+    <t>ONLY  P2 + P8</t>
+  </si>
+  <si>
+    <t>en attente de remplacement</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>P8</t>
+  </si>
+  <si>
+    <t>Mrs PINHEIRO</t>
+  </si>
+  <si>
+    <t>ONLY P6 TO P9</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>M LEDUC</t>
+  </si>
+  <si>
+    <t>M ROLL</t>
+  </si>
+  <si>
+    <t>ONLY P5 TO P9</t>
+  </si>
+  <si>
+    <t>M IONITA</t>
+  </si>
+  <si>
+    <t>Mrs ZARB HABER</t>
+  </si>
+  <si>
+    <t>ONLY P9</t>
+  </si>
+  <si>
+    <t>Mrs LE GOALLER</t>
+  </si>
+  <si>
     <t>12/6</t>
-  </si>
-  <si>
-    <t>Go to the library</t>
-  </si>
-  <si>
-    <t>P4/S3L1-SKA</t>
-  </si>
-  <si>
-    <t>Go to the libray</t>
-  </si>
-  <si>
-    <t>Mrs ZAJICKOVA</t>
-  </si>
-  <si>
-    <t>ONLY  P2 + P8</t>
-  </si>
-  <si>
-    <t>en attente de remplacement</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>P8</t>
-  </si>
-  <si>
-    <t>Mrs PINHEIRO</t>
-  </si>
-  <si>
-    <t>ONLY P6 TO P9</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>M LEDUC</t>
-  </si>
-  <si>
-    <t>M ROLL</t>
-  </si>
-  <si>
-    <t>ONLY P5 TO P9</t>
-  </si>
-  <si>
-    <t>M IONITA</t>
-  </si>
-  <si>
-    <t>Mrs ZARB HABER</t>
-  </si>
-  <si>
-    <t>ONLY P9</t>
-  </si>
-  <si>
-    <t>Mrs LE GOALLER</t>
   </si>
   <si>
     <t>Mrs NECHITA</t>
@@ -241,7 +277,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -273,6 +309,17 @@
       <color rgb="FF000000"/>
       <name val="Verdana"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Verdana"/>
     </font>
   </fonts>
   <fills count="3">
@@ -366,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -412,6 +459,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -736,7 +786,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -789,43 +839,43 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="36">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:12" ht="18">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="E3" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="5" t="s">
+    </row>
+    <row r="4" spans="1:12" ht="36">
+      <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:12" ht="36">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
+      <c r="B4" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="C4" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" spans="1:12" ht="18">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:12" ht="36">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:12" ht="18">
@@ -833,76 +883,72 @@
         <v>18</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>17</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>17</v>
+        <v>23</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>20</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>27</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="C11" s="15" t="s">
         <v>29</v>
@@ -915,81 +961,81 @@
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
+      <c r="A12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="C12" s="15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
       <c r="C13" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>37</v>
-      </c>
     </row>
     <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
+      <c r="A14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="C14" s="15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="15" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D15" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>41</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="15" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>45</v>
-      </c>
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
       <c r="C17" s="15" t="s">
         <v>46</v>
       </c>
@@ -997,15 +1043,15 @@
         <v>47</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18">
       <c r="A18" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>50</v>
@@ -1018,54 +1064,54 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="3"/>
-      <c r="B19" s="4"/>
+      <c r="A19" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="C19" s="15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="15" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>58</v>
+      <c r="A21" s="3"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="15" t="s">
+        <v>54</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>59</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18">
       <c r="A22" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>61</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>62</v>
@@ -1078,16 +1124,26 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="18">
-      <c r="A23" s="11"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
+      <c r="A23" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="24" spans="1:5" ht="18">
       <c r="A24" s="11"/>
       <c r="B24" s="12"/>
-      <c r="C24" s="13"/>
+      <c r="C24" s="14"/>
       <c r="D24" s="11"/>
       <c r="E24" s="11"/>
     </row>
@@ -1097,6 +1153,13 @@
       <c r="C25" s="13"/>
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
+    </row>
+    <row r="26" spans="1:5" ht="18">
+      <c r="A26" s="11"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-12 09:10
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10731" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7DFDC0C7-389B-4555-AA6C-DDF9167C9741}"/>
+  <xr:revisionPtr revIDLastSave="10740" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5AA0490-8749-4D37-BE10-6178DA0B5124}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="68">
   <si>
     <t>NOMS</t>
   </si>
@@ -111,13 +111,7 @@
     <t>ONLY  P2 + P8</t>
   </si>
   <si>
-    <t>en attente de remplacement</t>
-  </si>
-  <si>
-    <t>P2</t>
-  </si>
-  <si>
-    <t>P8</t>
+    <t>*</t>
   </si>
   <si>
     <t>Mrs PINHEIRO</t>
@@ -126,9 +120,6 @@
     <t>ONLY P6 TO P9</t>
   </si>
   <si>
-    <t>*</t>
-  </si>
-  <si>
     <t>M LEDUC</t>
   </si>
   <si>
@@ -147,6 +138,12 @@
     <t>ONLY P9</t>
   </si>
   <si>
+    <t>Mrs SCHALLHORN</t>
+  </si>
+  <si>
+    <t>ONLY P7 TO P9</t>
+  </si>
+  <si>
     <t>Mrs LE GOALLER</t>
   </si>
   <si>
@@ -165,7 +162,7 @@
     <t>Mrs GESTHUISEN</t>
   </si>
   <si>
-    <t>M. KLOPP</t>
+    <t>Mrs REYNAUD</t>
   </si>
   <si>
     <t>P4/S4L4-DEA</t>
@@ -852,7 +849,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="36">
+    <row r="4" spans="1:12" ht="18">
       <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
@@ -862,20 +859,20 @@
       <c r="C4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+    </row>
+    <row r="5" spans="1:12" ht="18">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" spans="1:12" ht="36">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
+      <c r="B5" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="C5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>17</v>
-      </c>
+      <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:12" ht="18">
@@ -883,261 +880,261 @@
         <v>18</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>20</v>
+        <v>17</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>15</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>26</v>
-      </c>
       <c r="C10" s="15" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="D11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="15" t="s">
+      <c r="D12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>37</v>
-      </c>
       <c r="E13" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="15" t="s">
+      <c r="D14" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3"/>
       <c r="B15" s="4"/>
       <c r="C15" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>43</v>
-      </c>
       <c r="E15" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
       <c r="C16" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="E16" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>47</v>
-      </c>
       <c r="E17" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="18">
       <c r="A18" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="C18" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="15" t="s">
+      <c r="D18" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="18">
       <c r="A19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C19" s="15" t="s">
+      <c r="D19" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="18">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>58</v>
-      </c>
       <c r="E20" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="18">
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="18">
       <c r="A22" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="C22" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="D22" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="18">
       <c r="A23" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C23" s="10" t="s">
+      <c r="D23" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>67</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18">

</xml_diff>

<commit_message>
MAJ absences 2026-06-15 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10740" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5AA0490-8749-4D37-BE10-6178DA0B5124}"/>
+  <xr:revisionPtr revIDLastSave="10746" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3ABF6C7-EEF9-424A-A52F-262FAD2F062D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,224 +57,89 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>Mrs KNIHAROVA</t>
-  </si>
-  <si>
-    <t>12/6 ONLY P1 TO P6</t>
-  </si>
-  <si>
-    <t>Mrs THEODOROU</t>
-  </si>
-  <si>
-    <t>P4/S3L1-SKA</t>
-  </si>
-  <si>
-    <t>Go to the libray</t>
-  </si>
-  <si>
-    <t>Mrs JUHASZ</t>
-  </si>
-  <si>
-    <t>P6/S1L1-SKA</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Verdana"/>
-      </rPr>
-      <t>C10</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Verdana"/>
-      </rPr>
-      <t>6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Verdana"/>
-      </rPr>
-      <t xml:space="preserve">   attention!</t>
-    </r>
-  </si>
-  <si>
-    <t>Mrs ZAJICKOVA</t>
-  </si>
-  <si>
-    <t>ONLY  P2 + P8</t>
+    <t>M. WAECHTER</t>
+  </si>
+  <si>
+    <t>15/6 ONLY P5 TO P9</t>
+  </si>
+  <si>
+    <t>M. BERNET</t>
+  </si>
+  <si>
+    <t>P1/S6CHI-FRB</t>
+  </si>
+  <si>
+    <t>D306</t>
+  </si>
+  <si>
+    <t>P2/S6CHI-FRB</t>
+  </si>
+  <si>
+    <t>P3/S4PHY-FRA</t>
+  </si>
+  <si>
+    <t>Mrs COQUELIN</t>
+  </si>
+  <si>
+    <t>P5/S5CHI-FRD</t>
+  </si>
+  <si>
+    <t>MRS ORMASTI</t>
+  </si>
+  <si>
+    <t>ONLY P5 TO P9</t>
+  </si>
+  <si>
+    <t>Mrs STRAUS ZULU</t>
+  </si>
+  <si>
+    <t>P5/S4GEO-FRB</t>
+  </si>
+  <si>
+    <t>A001</t>
+  </si>
+  <si>
+    <t>Mrs IANNOPOLLO</t>
   </si>
   <si>
     <t>*</t>
   </si>
   <si>
-    <t>Mrs PINHEIRO</t>
+    <t>Mrs TABONE</t>
+  </si>
+  <si>
+    <t>ONLY P6 TO P7</t>
+  </si>
+  <si>
+    <t>Mrs BUNDARA</t>
+  </si>
+  <si>
+    <t>P6/S3L1-ENA</t>
+  </si>
+  <si>
+    <t>A108</t>
+  </si>
+  <si>
+    <t>Mrs DUFF</t>
+  </si>
+  <si>
+    <t>P7/S2L1-ENB</t>
+  </si>
+  <si>
+    <t>B104</t>
+  </si>
+  <si>
+    <t>Mr ANDERSSON</t>
   </si>
   <si>
     <t>ONLY P6 TO P9</t>
-  </si>
-  <si>
-    <t>M LEDUC</t>
-  </si>
-  <si>
-    <t>M ROLL</t>
-  </si>
-  <si>
-    <t>ONLY P5 TO P9</t>
-  </si>
-  <si>
-    <t>M IONITA</t>
-  </si>
-  <si>
-    <t>Mrs ZARB HABER</t>
-  </si>
-  <si>
-    <t>ONLY P9</t>
-  </si>
-  <si>
-    <t>Mrs SCHALLHORN</t>
-  </si>
-  <si>
-    <t>ONLY P7 TO P9</t>
-  </si>
-  <si>
-    <t>Mrs LE GOALLER</t>
-  </si>
-  <si>
-    <t>12/6</t>
-  </si>
-  <si>
-    <t>Mrs NECHITA</t>
-  </si>
-  <si>
-    <t>P5/S2L2-DEA</t>
-  </si>
-  <si>
-    <t>B217</t>
-  </si>
-  <si>
-    <t>Mrs GESTHUISEN</t>
-  </si>
-  <si>
-    <t>Mrs REYNAUD</t>
-  </si>
-  <si>
-    <t>P4/S4L4-DEA</t>
-  </si>
-  <si>
-    <t>C110</t>
-  </si>
-  <si>
-    <t>Mrs CASTELLO</t>
-  </si>
-  <si>
-    <t>P5/S4L4-DEA</t>
-  </si>
-  <si>
-    <t>Mrs VORNICESCU</t>
-  </si>
-  <si>
-    <t>Mrs MONTEIRO</t>
-  </si>
-  <si>
-    <t>P2/S4XMADEA</t>
-  </si>
-  <si>
-    <t>D312</t>
-  </si>
-  <si>
-    <t>M HENTSCHEL</t>
-  </si>
-  <si>
-    <t>P4/S5PHYDEA</t>
-  </si>
-  <si>
-    <t>M. CHEILAS</t>
-  </si>
-  <si>
-    <t>P7/S2MATDEB</t>
-  </si>
-  <si>
-    <t>MRS MYSIRLAKI</t>
-  </si>
-  <si>
-    <t>P8/S5MA6DEA</t>
-  </si>
-  <si>
-    <t>M CHEILAS</t>
-  </si>
-  <si>
-    <t>ONLY P1</t>
-  </si>
-  <si>
-    <t>M ZAHARIA</t>
-  </si>
-  <si>
-    <t>P1/S1SCI-ENB</t>
-  </si>
-  <si>
-    <t>D204</t>
-  </si>
-  <si>
-    <t>Mrs ORMASTI</t>
-  </si>
-  <si>
-    <t>M. GILLIG</t>
-  </si>
-  <si>
-    <t>P1/S1SCH-FRA</t>
-  </si>
-  <si>
-    <t>A001</t>
-  </si>
-  <si>
-    <t>M. SNAPPE</t>
-  </si>
-  <si>
-    <t>P2/S1SCH-FRA</t>
-  </si>
-  <si>
-    <t>P7/S1SCH-FRB</t>
-  </si>
-  <si>
-    <t>Mrs FORET-TOUSSAINT</t>
-  </si>
-  <si>
-    <t>ONLY P3</t>
-  </si>
-  <si>
-    <t>Mr BERRICHI</t>
-  </si>
-  <si>
-    <t>P3/S2MOR-FRC</t>
-  </si>
-  <si>
-    <t>B206</t>
-  </si>
-  <si>
-    <t>Mrs DI SALVATORE</t>
-  </si>
-  <si>
-    <t>Mrs GALEZIOK</t>
-  </si>
-  <si>
-    <t>P3/S2RCA-FRA</t>
-  </si>
-  <si>
-    <t>A003</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -306,17 +171,6 @@
       <color rgb="FF000000"/>
       <name val="Verdana"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Verdana"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Verdana"/>
     </font>
   </fonts>
   <fills count="3">
@@ -410,7 +264,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -456,9 +310,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -783,7 +634,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -840,63 +691,67 @@
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="18">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E4" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="18">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="10" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="18">
-      <c r="A4" s="3" t="s">
+      <c r="D5" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" spans="1:12" ht="18">
-      <c r="A5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="E5" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="18">
       <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>15</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
@@ -906,257 +761,64 @@
         <v>21</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>22</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="A11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>34</v>
-      </c>
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="18">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="18">
-      <c r="A22" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="18">
-      <c r="A23" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="18">
-      <c r="A24" s="11"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-    </row>
-    <row r="25" spans="1:5" ht="18">
-      <c r="A25" s="11"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-    </row>
-    <row r="26" spans="1:5" ht="18">
-      <c r="A26" s="11"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="11"/>
-      <c r="E26" s="11"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1166,30 +828,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1487,8 +1125,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1496,5 +1158,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-15 08:20
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10746" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3ABF6C7-EEF9-424A-A52F-262FAD2F062D}"/>
+  <xr:revisionPtr revIDLastSave="10764" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34A947B6-7A71-4571-8968-5E39E1BD590D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="toShow">Feuil1!$A:$E</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
-    <definedName name="toShow">Feuil1!$A:$E</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
   <si>
     <t>NOMS</t>
   </si>
@@ -127,6 +127,42 @@
   </si>
   <si>
     <t>B104</t>
+  </si>
+  <si>
+    <t>MRS SORENSEN</t>
+  </si>
+  <si>
+    <t>15/06</t>
+  </si>
+  <si>
+    <t>MR KARAGIANNIDIS</t>
+  </si>
+  <si>
+    <t>P1/S2MATENB</t>
+  </si>
+  <si>
+    <t>A007</t>
+  </si>
+  <si>
+    <t>MR LIPPERT</t>
+  </si>
+  <si>
+    <t>P2/S4MA4ENA</t>
+  </si>
+  <si>
+    <t>MRS DROSOFORIDOU</t>
+  </si>
+  <si>
+    <t>P3/S4MA4ENA</t>
+  </si>
+  <si>
+    <t>MRS SADELER</t>
+  </si>
+  <si>
+    <t>P6/S2MATDAA</t>
+  </si>
+  <si>
+    <t>C203</t>
   </si>
   <si>
     <t>Mr ANDERSSON</t>
@@ -634,7 +670,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -793,32 +829,88 @@
       <c r="B10" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="11"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -828,6 +920,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1125,32 +1241,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1158,5 +1250,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-15 08:35
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10764" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34A947B6-7A71-4571-8968-5E39E1BD590D}"/>
+  <xr:revisionPtr revIDLastSave="10765" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AF6F0B-4995-4360-8CB3-FEE75A6B650F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
     <definedName name="toShow">Feuil1!$A:$E</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -165,7 +165,7 @@
     <t>C203</t>
   </si>
   <si>
-    <t>Mr ANDERSSON</t>
+    <t>MRS ANDERSSON</t>
   </si>
   <si>
     <t>ONLY P6 TO P9</t>
@@ -920,15 +920,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -941,6 +932,15 @@
     <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1242,11 +1242,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-15 08:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10765" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0AF6F0B-4995-4360-8CB3-FEE75A6B650F}"/>
+  <xr:revisionPtr revIDLastSave="10772" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E148C95-05BD-411A-9497-FE5E109F0C85}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="48">
   <si>
     <t>NOMS</t>
   </si>
@@ -163,6 +163,21 @@
   </si>
   <si>
     <t>C203</t>
+  </si>
+  <si>
+    <t>MRS FORÊT</t>
+  </si>
+  <si>
+    <t>ONLY P4</t>
+  </si>
+  <si>
+    <t>MR DALGAS</t>
+  </si>
+  <si>
+    <t>P4/S2MORFRC</t>
+  </si>
+  <si>
+    <t>B206</t>
   </si>
   <si>
     <t>MRS ANDERSSON</t>
@@ -670,7 +685,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -885,23 +900,33 @@
       <c r="B14" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="11"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="11"/>
       <c r="B16" s="12"/>
-      <c r="C16" s="13"/>
+      <c r="C16" s="14"/>
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
     </row>
@@ -911,6 +936,13 @@
       <c r="C17" s="13"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="11"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -920,30 +952,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1241,8 +1249,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1250,5 +1282,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-15 12:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10772" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E148C95-05BD-411A-9497-FE5E109F0C85}"/>
+  <xr:revisionPtr revIDLastSave="10774" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA0AF7FB-F390-4407-8C65-B652CCF50B63}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
   <si>
     <t>NOMS</t>
   </si>
@@ -90,19 +90,10 @@
     <t>ONLY P5 TO P9</t>
   </si>
   <si>
-    <t>Mrs STRAUS ZULU</t>
-  </si>
-  <si>
-    <t>P5/S4GEO-FRB</t>
-  </si>
-  <si>
-    <t>A001</t>
+    <t>*</t>
   </si>
   <si>
     <t>Mrs IANNOPOLLO</t>
-  </si>
-  <si>
-    <t>*</t>
   </si>
   <si>
     <t>Mrs TABONE</t>
@@ -787,138 +778,134 @@
       <c r="C6" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>18</v>
-      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="10" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="E10" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="10" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="10" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>42</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
@@ -952,6 +939,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1249,15 +1245,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1274,11 +1261,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-15 12:40
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10774" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FA0AF7FB-F390-4407-8C65-B652CCF50B63}"/>
+  <xr:revisionPtr revIDLastSave="10784" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D6945EF-F748-4BD1-B7DD-FD2990741C2F}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
   <si>
     <t>NOMS</t>
   </si>
@@ -175,6 +175,24 @@
   </si>
   <si>
     <t>ONLY P6 TO P9</t>
+  </si>
+  <si>
+    <t>MRS PRIESS</t>
+  </si>
+  <si>
+    <t>MR BLOND</t>
+  </si>
+  <si>
+    <t>P6/S1ART--E</t>
+  </si>
+  <si>
+    <t>A302</t>
+  </si>
+  <si>
+    <t>MRS FRYGANA</t>
+  </si>
+  <si>
+    <t>P7/S1ART--E</t>
   </si>
 </sst>
 </file>
@@ -306,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -336,18 +354,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -676,7 +682,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -904,32 +910,41 @@
       <c r="B15" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C15" s="15" t="s">
+      <c r="C15" s="11" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
+      <c r="A16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="11"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="11"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>48</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -939,15 +954,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1245,6 +1251,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1261,11 +1276,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-15 16:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10784" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D6945EF-F748-4BD1-B7DD-FD2990741C2F}"/>
+  <xr:revisionPtr revIDLastSave="10788" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{060C361F-6307-4256-87E7-8307DBD022D8}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
   <si>
     <t>NOMS</t>
   </si>
@@ -154,6 +154,9 @@
   </si>
   <si>
     <t>C203</t>
+  </si>
+  <si>
+    <t>MR CASTANET</t>
   </si>
   <si>
     <t>MRS FORÊT</t>
@@ -682,7 +685,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -891,59 +894,72 @@
         <v>38</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>42</v>
-      </c>
+        <v>16</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="C16" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" s="5" t="s">
+      <c r="C17" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="10" t="s">
+      <c r="E17" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="5" t="s">
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>48</v>
+      <c r="D18" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -954,6 +970,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1251,15 +1276,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1276,11 +1292,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-15 16:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10788" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{060C361F-6307-4256-87E7-8307DBD022D8}"/>
+  <xr:revisionPtr revIDLastSave="10791" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B7E87AE-6AF4-4798-A62B-A18FFDC9D066}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,145 +57,10 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>M. WAECHTER</t>
-  </si>
-  <si>
-    <t>15/6 ONLY P5 TO P9</t>
-  </si>
-  <si>
-    <t>M. BERNET</t>
-  </si>
-  <si>
-    <t>P1/S6CHI-FRB</t>
-  </si>
-  <si>
-    <t>D306</t>
-  </si>
-  <si>
-    <t>P2/S6CHI-FRB</t>
-  </si>
-  <si>
-    <t>P3/S4PHY-FRA</t>
-  </si>
-  <si>
-    <t>Mrs COQUELIN</t>
-  </si>
-  <si>
-    <t>P5/S5CHI-FRD</t>
-  </si>
-  <si>
-    <t>MRS ORMASTI</t>
-  </si>
-  <si>
-    <t>ONLY P5 TO P9</t>
-  </si>
-  <si>
     <t>*</t>
   </si>
   <si>
-    <t>Mrs IANNOPOLLO</t>
-  </si>
-  <si>
-    <t>Mrs TABONE</t>
-  </si>
-  <si>
-    <t>ONLY P6 TO P7</t>
-  </si>
-  <si>
-    <t>Mrs BUNDARA</t>
-  </si>
-  <si>
-    <t>P6/S3L1-ENA</t>
-  </si>
-  <si>
-    <t>A108</t>
-  </si>
-  <si>
-    <t>Mrs DUFF</t>
-  </si>
-  <si>
-    <t>P7/S2L1-ENB</t>
-  </si>
-  <si>
-    <t>B104</t>
-  </si>
-  <si>
-    <t>MRS SORENSEN</t>
-  </si>
-  <si>
-    <t>15/06</t>
-  </si>
-  <si>
-    <t>MR KARAGIANNIDIS</t>
-  </si>
-  <si>
-    <t>P1/S2MATENB</t>
-  </si>
-  <si>
-    <t>A007</t>
-  </si>
-  <si>
-    <t>MR LIPPERT</t>
-  </si>
-  <si>
-    <t>P2/S4MA4ENA</t>
-  </si>
-  <si>
-    <t>MRS DROSOFORIDOU</t>
-  </si>
-  <si>
-    <t>P3/S4MA4ENA</t>
-  </si>
-  <si>
-    <t>MRS SADELER</t>
-  </si>
-  <si>
-    <t>P6/S2MATDAA</t>
-  </si>
-  <si>
-    <t>C203</t>
-  </si>
-  <si>
-    <t>MR CASTANET</t>
-  </si>
-  <si>
-    <t>MRS FORÊT</t>
-  </si>
-  <si>
-    <t>ONLY P4</t>
-  </si>
-  <si>
-    <t>MR DALGAS</t>
-  </si>
-  <si>
-    <t>P4/S2MORFRC</t>
-  </si>
-  <si>
-    <t>B206</t>
-  </si>
-  <si>
-    <t>MRS ANDERSSON</t>
-  </si>
-  <si>
-    <t>ONLY P6 TO P9</t>
-  </si>
-  <si>
-    <t>MRS PRIESS</t>
-  </si>
-  <si>
-    <t>MR BLOND</t>
-  </si>
-  <si>
-    <t>P6/S1ART--E</t>
-  </si>
-  <si>
-    <t>A302</t>
-  </si>
-  <si>
-    <t>MRS FRYGANA</t>
-  </si>
-  <si>
-    <t>P7/S1ART--E</t>
+    <t>16/06</t>
   </si>
 </sst>
 </file>
@@ -728,239 +593,121 @@
       <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C2" s="10"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:12" ht="18">
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
-      <c r="C3" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
     </row>
     <row r="4" spans="1:12" ht="18">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
-      <c r="C4" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
-      <c r="C5" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>16</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="10"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>16</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>22</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
-      <c r="C9" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>25</v>
-      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>30</v>
-      </c>
+      <c r="C12" s="10"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>37</v>
-      </c>
+      <c r="C13" s="10"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>16</v>
-      </c>
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="10"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>43</v>
-      </c>
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
     </row>
     <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>49</v>
-      </c>
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
     </row>
     <row r="18" spans="1:5" ht="18">
       <c r="A18" s="3"/>
       <c r="B18" s="4"/>
-      <c r="C18" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>49</v>
-      </c>
+      <c r="C18" s="10"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -970,12 +717,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1277,22 +1030,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1300,5 +1047,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-16 08:35
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10791" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B7E87AE-6AF4-4798-A62B-A18FFDC9D066}"/>
+  <xr:revisionPtr revIDLastSave="10798" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BEFCF84-72A9-4AA7-9A9F-71A3B413EB3B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,10 +57,25 @@
     <t>SALLES</t>
   </si>
   <si>
+    <t>MRS TOPAL</t>
+  </si>
+  <si>
+    <t>16/06</t>
+  </si>
+  <si>
+    <t>MR MULRENNAN</t>
+  </si>
+  <si>
+    <t>P4/S4ECOENC</t>
+  </si>
+  <si>
+    <t>C001</t>
+  </si>
+  <si>
+    <t>MRS PETROULI</t>
+  </si>
+  <si>
     <t>*</t>
-  </si>
-  <si>
-    <t>16/06</t>
   </si>
 </sst>
 </file>
@@ -593,14 +608,26 @@
       <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="C2" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="18">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="10"/>
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>11</v>
+      </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
@@ -717,21 +744,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1029,6 +1041,21 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1039,11 +1066,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-16 16:35
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10798" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BEFCF84-72A9-4AA7-9A9F-71A3B413EB3B}"/>
+  <xr:revisionPtr revIDLastSave="10801" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF9BA9CE-D78E-4468-83C1-760E33B39318}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,25 +57,55 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MRS TOPAL</t>
-  </si>
-  <si>
-    <t>16/06</t>
-  </si>
-  <si>
-    <t>MR MULRENNAN</t>
-  </si>
-  <si>
-    <t>P4/S4ECOENC</t>
-  </si>
-  <si>
-    <t>C001</t>
-  </si>
-  <si>
-    <t>MRS PETROULI</t>
-  </si>
-  <si>
-    <t>*</t>
+    <t>MR COUCHE</t>
+  </si>
+  <si>
+    <t>ONLY P7</t>
+  </si>
+  <si>
+    <t>MRS PAVLIDOU</t>
+  </si>
+  <si>
+    <t>P7/S4CHIFRB</t>
+  </si>
+  <si>
+    <t>D304</t>
+  </si>
+  <si>
+    <t>MR KUPPER</t>
+  </si>
+  <si>
+    <t>17/06</t>
+  </si>
+  <si>
+    <t>MR PRIESS J</t>
+  </si>
+  <si>
+    <t>P4/S2L1-DEA</t>
+  </si>
+  <si>
+    <t>C111</t>
+  </si>
+  <si>
+    <t>MRS BENETTI</t>
+  </si>
+  <si>
+    <t>MRS GARIOU</t>
+  </si>
+  <si>
+    <t>P2/S1L1-ITB</t>
+  </si>
+  <si>
+    <t>C101</t>
+  </si>
+  <si>
+    <t>MRS PRIESS N</t>
+  </si>
+  <si>
+    <t>P7/S4L1-ITA</t>
+  </si>
+  <si>
+    <t>B116</t>
   </si>
 </sst>
 </file>
@@ -116,18 +146,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -207,7 +231,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -237,9 +261,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -565,7 +586,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -623,27 +644,47 @@
         <v>10</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+        <v>12</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4" spans="1:12" ht="18">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="C5" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="6" spans="1:12" ht="18">
       <c r="A6" s="3"/>
@@ -651,90 +692,6 @@
       <c r="C6" s="10"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
-    </row>
-    <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-    </row>
-    <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -744,6 +701,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1041,21 +1013,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1066,11 +1023,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-17 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10801" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF9BA9CE-D78E-4468-83C1-760E33B39318}"/>
+  <xr:revisionPtr revIDLastSave="10827" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{517C7B24-5416-4E04-A87B-098ED084C407}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="toShow">Feuil1!$A:$E</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
-    <definedName name="toShow">Feuil1!$A:$E</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
   <si>
     <t>NOMS</t>
   </si>
@@ -106,6 +106,45 @@
   </si>
   <si>
     <t>B116</t>
+  </si>
+  <si>
+    <t>MRS VEHLING</t>
+  </si>
+  <si>
+    <t>MRS PETROULI</t>
+  </si>
+  <si>
+    <t>P1/S2SCHDEB</t>
+  </si>
+  <si>
+    <t>C107</t>
+  </si>
+  <si>
+    <t>MR KLUPPELHOLZ</t>
+  </si>
+  <si>
+    <t>P3/S2L3DEB</t>
+  </si>
+  <si>
+    <t>B004</t>
+  </si>
+  <si>
+    <t>MRS HERRIG</t>
+  </si>
+  <si>
+    <t>P5/S1L2DEB</t>
+  </si>
+  <si>
+    <t>MRS RIBA</t>
+  </si>
+  <si>
+    <t>P6/S1L2DEB</t>
+  </si>
+  <si>
+    <t>MRS LEDUC</t>
+  </si>
+  <si>
+    <t>P7/S1L2DEB</t>
   </si>
 </sst>
 </file>
@@ -586,7 +625,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -687,11 +726,80 @@
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="18">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="18">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="18">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="18">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -701,21 +809,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1013,7 +1106,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1022,14 +1115,29 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-17 08:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10827" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{517C7B24-5416-4E04-A87B-098ED084C407}"/>
+  <xr:revisionPtr revIDLastSave="10831" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82E4AA67-EAB4-4446-B599-39B276124244}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
   <si>
     <t>NOMS</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>P7/S1L2DEB</t>
+  </si>
+  <si>
+    <t>MRS OSKARSDOTTIR</t>
   </si>
 </sst>
 </file>
@@ -625,7 +628,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -795,11 +798,29 @@
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>11</v>
+      </c>
       <c r="C11" s="10"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -809,6 +830,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1106,32 +1151,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1139,5 +1160,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-17 08:10
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10831" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82E4AA67-EAB4-4446-B599-39B276124244}"/>
+  <xr:revisionPtr revIDLastSave="10837" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30BE6B8E-0D66-430D-A4D5-AB2C49840018}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
   <si>
     <t>NOMS</t>
   </si>
@@ -148,6 +148,21 @@
   </si>
   <si>
     <t>MRS OSKARSDOTTIR</t>
+  </si>
+  <si>
+    <t>MRS RHEINHEIMER</t>
+  </si>
+  <si>
+    <t>P1/S4ECOENB</t>
+  </si>
+  <si>
+    <t>B015</t>
+  </si>
+  <si>
+    <t>MRS REBERSAK</t>
+  </si>
+  <si>
+    <t>P2/S4ECOENB</t>
   </si>
 </sst>
 </file>
@@ -804,16 +819,28 @@
       <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="C11" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="C12" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-17 09:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10837" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30BE6B8E-0D66-430D-A4D5-AB2C49840018}"/>
+  <xr:revisionPtr revIDLastSave="10838" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7A25251-CD7E-4D69-B295-0292B7B10275}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
     <definedName name="toShow">Feuil1!$A:$E</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
   <si>
     <t>NOMS</t>
   </si>
@@ -117,22 +117,25 @@
     <t>P1/S2SCHDEB</t>
   </si>
   <si>
+    <t>B011</t>
+  </si>
+  <si>
+    <t>MR KLUPPELHOLZ</t>
+  </si>
+  <si>
+    <t>P3/S2L3DEB</t>
+  </si>
+  <si>
+    <t>B004</t>
+  </si>
+  <si>
+    <t>MRS HERRIG</t>
+  </si>
+  <si>
+    <t>P5/S1L2DEB</t>
+  </si>
+  <si>
     <t>C107</t>
-  </si>
-  <si>
-    <t>MR KLUPPELHOLZ</t>
-  </si>
-  <si>
-    <t>P3/S2L3DEB</t>
-  </si>
-  <si>
-    <t>B004</t>
-  </si>
-  <si>
-    <t>MRS HERRIG</t>
-  </si>
-  <si>
-    <t>P5/S1L2DEB</t>
   </si>
   <si>
     <t>MRS RIBA</t>
@@ -783,63 +786,63 @@
         <v>30</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
@@ -857,30 +860,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1178,8 +1157,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1187,5 +1190,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-17 12:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10838" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7A25251-CD7E-4D69-B295-0292B7B10275}"/>
+  <xr:revisionPtr revIDLastSave="10839" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E09E7831-8FC2-4557-9608-AF1C2649180C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -132,7 +132,7 @@
     <t>MRS HERRIG</t>
   </si>
   <si>
-    <t>P5/S1L2DEB</t>
+    <t>P5/S3L3DEA</t>
   </si>
   <si>
     <t>C107</t>
@@ -860,6 +860,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1157,32 +1181,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1190,5 +1190,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-17 12:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10839" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E09E7831-8FC2-4557-9608-AF1C2649180C}"/>
+  <xr:revisionPtr revIDLastSave="10840" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E734C38B-4DB2-485A-99CB-F62BC8149490}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -138,7 +138,7 @@
     <t>C107</t>
   </si>
   <si>
-    <t>MRS RIBA</t>
+    <t>MR NEMEC</t>
   </si>
   <si>
     <t>P6/S1L2DEB</t>
@@ -860,30 +860,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1181,8 +1157,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1190,5 +1190,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-17 15:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10840" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E734C38B-4DB2-485A-99CB-F62BC8149490}"/>
+  <xr:revisionPtr revIDLastSave="10842" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4293521-8361-4CF6-9C25-51C6C7824143}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,115 +57,151 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MR COUCHE</t>
-  </si>
-  <si>
-    <t>ONLY P7</t>
-  </si>
-  <si>
-    <t>MRS PAVLIDOU</t>
-  </si>
-  <si>
-    <t>P7/S4CHIFRB</t>
-  </si>
-  <si>
-    <t>D304</t>
+    <t>MRS VEHLING</t>
+  </si>
+  <si>
+    <t>18/02</t>
+  </si>
+  <si>
+    <t>MRS NECHITA</t>
+  </si>
+  <si>
+    <t>P1/S3SCHDEA</t>
+  </si>
+  <si>
+    <t>B017</t>
+  </si>
+  <si>
+    <t>MRS DEMARTINI</t>
+  </si>
+  <si>
+    <t>P2/S1SCHENC</t>
+  </si>
+  <si>
+    <t>B216</t>
+  </si>
+  <si>
+    <t>MRS DIMMOCK</t>
+  </si>
+  <si>
+    <t>P3/S1L2-DEB</t>
+  </si>
+  <si>
+    <t>C107</t>
+  </si>
+  <si>
+    <t>MR KARAGIANNIS</t>
+  </si>
+  <si>
+    <t>P4/S1L2-DEB</t>
+  </si>
+  <si>
+    <t>MRS LÜDERS</t>
+  </si>
+  <si>
+    <t>P8/S2L3-DEB</t>
+  </si>
+  <si>
+    <t>B004</t>
+  </si>
+  <si>
+    <t>MRS KRALJIC</t>
+  </si>
+  <si>
+    <t>MRS RAYMONDAUD</t>
+  </si>
+  <si>
+    <t>P1/S4L3-FRA</t>
+  </si>
+  <si>
+    <t>B211</t>
+  </si>
+  <si>
+    <t>MRS NOBIS</t>
+  </si>
+  <si>
+    <t>P2/S3L2-FRC</t>
+  </si>
+  <si>
+    <t>B106</t>
+  </si>
+  <si>
+    <t>MRS DESROSIERS</t>
+  </si>
+  <si>
+    <t>P3/S1L2-FRB</t>
+  </si>
+  <si>
+    <t>MRS DI SALVATORE</t>
+  </si>
+  <si>
+    <t>P4/S1L2-FRB</t>
+  </si>
+  <si>
+    <t>MRS GROBER</t>
+  </si>
+  <si>
+    <t>ONLY P2 TO P8</t>
+  </si>
+  <si>
+    <t>MRS POTIN</t>
+  </si>
+  <si>
+    <t>P3/S1L2-FRA</t>
+  </si>
+  <si>
+    <t>D106</t>
+  </si>
+  <si>
+    <t>MR HADJI</t>
+  </si>
+  <si>
+    <t>P4/S1L2-FRA</t>
   </si>
   <si>
     <t>MR KUPPER</t>
   </si>
   <si>
-    <t>17/06</t>
-  </si>
-  <si>
-    <t>MR PRIESS J</t>
-  </si>
-  <si>
-    <t>P4/S2L1-DEA</t>
-  </si>
-  <si>
-    <t>C111</t>
-  </si>
-  <si>
-    <t>MRS BENETTI</t>
-  </si>
-  <si>
-    <t>MRS GARIOU</t>
-  </si>
-  <si>
-    <t>P2/S1L1-ITB</t>
-  </si>
-  <si>
-    <t>C101</t>
-  </si>
-  <si>
-    <t>MRS PRIESS N</t>
-  </si>
-  <si>
-    <t>P7/S4L1-ITA</t>
-  </si>
-  <si>
-    <t>B116</t>
-  </si>
-  <si>
-    <t>MRS VEHLING</t>
-  </si>
-  <si>
-    <t>MRS PETROULI</t>
-  </si>
-  <si>
-    <t>P1/S2SCHDEB</t>
-  </si>
-  <si>
-    <t>B011</t>
-  </si>
-  <si>
-    <t>MR KLUPPELHOLZ</t>
-  </si>
-  <si>
-    <t>P3/S2L3DEB</t>
-  </si>
-  <si>
-    <t>B004</t>
-  </si>
-  <si>
-    <t>MRS HERRIG</t>
-  </si>
-  <si>
-    <t>P5/S3L3DEA</t>
-  </si>
-  <si>
-    <t>C107</t>
-  </si>
-  <si>
-    <t>MR NEMEC</t>
-  </si>
-  <si>
-    <t>P6/S1L2DEB</t>
-  </si>
-  <si>
-    <t>MRS LEDUC</t>
-  </si>
-  <si>
-    <t>P7/S1L2DEB</t>
-  </si>
-  <si>
-    <t>MRS OSKARSDOTTIR</t>
-  </si>
-  <si>
-    <t>MRS RHEINHEIMER</t>
-  </si>
-  <si>
-    <t>P1/S4ECOENB</t>
-  </si>
-  <si>
-    <t>B015</t>
-  </si>
-  <si>
-    <t>MRS REBERSAK</t>
-  </si>
-  <si>
-    <t>P2/S4ECOENB</t>
+    <t>P5/S3LATDEA</t>
+  </si>
+  <si>
+    <t>MR ROLL</t>
+  </si>
+  <si>
+    <t>P8/S2L3-FRA</t>
+  </si>
+  <si>
+    <t>D105</t>
+  </si>
+  <si>
+    <t>MRS PIERSON</t>
+  </si>
+  <si>
+    <t>MRS GRIRA</t>
+  </si>
+  <si>
+    <t>P5/S1L1-FRC</t>
+  </si>
+  <si>
+    <t>C202</t>
+  </si>
+  <si>
+    <t>MRS SADELER</t>
+  </si>
+  <si>
+    <t>P8/S4LATFRA</t>
+  </si>
+  <si>
+    <t>MR BOTH</t>
+  </si>
+  <si>
+    <t>MR BAZIN</t>
+  </si>
+  <si>
+    <t>P2/S4L1-ROA</t>
+  </si>
+  <si>
+    <t>B210</t>
   </si>
 </sst>
 </file>
@@ -646,7 +682,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -700,157 +736,222 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="18">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="E3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="5" t="s">
+    </row>
+    <row r="4" spans="1:12" ht="18">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" ht="18">
-      <c r="A4" s="3" t="s">
+      <c r="E4" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="18">
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="5" t="s">
+    </row>
+    <row r="7" spans="1:12" ht="18">
+      <c r="A7" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3" t="s">
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="D7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>24</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="10" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="10" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="C13" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -860,6 +961,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1157,15 +1267,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1182,11 +1283,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-18 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10842" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4293521-8361-4CF6-9C25-51C6C7824143}"/>
+  <xr:revisionPtr revIDLastSave="10874" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C217E3F-5B40-48C7-B7B7-560BEDA9E221}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="toShow">Feuil1!$A:$E</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
-    <definedName name="toShow">Feuil1!$A:$E</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="72">
   <si>
     <t>NOMS</t>
   </si>
@@ -202,6 +202,60 @@
   </si>
   <si>
     <t>B210</t>
+  </si>
+  <si>
+    <t>MRS OSKARSDOTTIR</t>
+  </si>
+  <si>
+    <t>18/06</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>MR PRIESS</t>
+  </si>
+  <si>
+    <t>MR THOUVENEL</t>
+  </si>
+  <si>
+    <t>P1/S1SCHDEA</t>
+  </si>
+  <si>
+    <t>B117</t>
+  </si>
+  <si>
+    <t>MRS PAVLIDOU</t>
+  </si>
+  <si>
+    <t>P2/S1SCHDEA</t>
+  </si>
+  <si>
+    <t>MRS WUTTKE</t>
+  </si>
+  <si>
+    <t>P3/S4HISDEA</t>
+  </si>
+  <si>
+    <t>MRS COSTESCU</t>
+  </si>
+  <si>
+    <t>GO TO LIBRARY</t>
+  </si>
+  <si>
+    <t>P5/S1L1ROA</t>
+  </si>
+  <si>
+    <t>MRS TOURA</t>
+  </si>
+  <si>
+    <t>P3/S2SCIELA</t>
+  </si>
+  <si>
+    <t>D210</t>
+  </si>
+  <si>
+    <t>MRS PETROULI</t>
   </si>
 </sst>
 </file>
@@ -682,7 +736,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U25"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -947,11 +1001,110 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="10"/>
+      <c r="A18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>56</v>
+      </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
+    </row>
+    <row r="19" spans="1:5" ht="18">
+      <c r="A19" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="18">
+      <c r="A20" s="3"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="18">
+      <c r="A21" s="3"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18">
+      <c r="A22" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="5"/>
+    </row>
+    <row r="23" spans="1:5" ht="18">
+      <c r="A23" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="18">
+      <c r="A24" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="10"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+    </row>
+    <row r="25" spans="1:5" ht="18">
+      <c r="A25" s="3"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -961,6 +1114,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -969,7 +1137,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1267,29 +1435,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-18 08:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10874" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C217E3F-5B40-48C7-B7B7-560BEDA9E221}"/>
+  <xr:revisionPtr revIDLastSave="10875" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{019026B0-C920-451E-BDCF-E616A0F3DFE5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
   <si>
     <t>NOMS</t>
   </si>
@@ -1095,7 +1095,9 @@
       <c r="B24" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="10"/>
+      <c r="C24" s="10" t="s">
+        <v>56</v>
+      </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
     </row>

</xml_diff>

<commit_message>
MAJ absences 2026-06-18 08:40
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10875" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{019026B0-C920-451E-BDCF-E616A0F3DFE5}"/>
+  <xr:revisionPtr revIDLastSave="10879" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74741822-8DC5-4258-B3D8-83887E0E6D45}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
     <definedName name="toShow">Feuil1!$A:$E</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
   <si>
     <t>NOMS</t>
   </si>
@@ -81,7 +81,7 @@
     <t>B216</t>
   </si>
   <si>
-    <t>MRS DIMMOCK</t>
+    <t>MR ZULU</t>
   </si>
   <si>
     <t>P3/S1L2-DEB</t>
@@ -256,6 +256,12 @@
   </si>
   <si>
     <t>MRS PETROULI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MR GILLIG </t>
+  </si>
+  <si>
+    <t>ONLY P1</t>
   </si>
 </sst>
 </file>
@@ -1102,9 +1108,15 @@
       <c r="E24" s="5"/>
     </row>
     <row r="25" spans="1:5" ht="18">
-      <c r="A25" s="3"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="10"/>
+      <c r="A25" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>56</v>
+      </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
     </row>
@@ -1116,21 +1128,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -1139,7 +1136,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1437,14 +1434,29 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-18 08:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10879" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74741822-8DC5-4258-B3D8-83887E0E6D45}"/>
+  <xr:revisionPtr revIDLastSave="10880" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFED1F84-82FD-4C60-81A8-11D15608395C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
   <si>
     <t>NOMS</t>
   </si>
@@ -216,16 +216,13 @@
     <t>MR PRIESS</t>
   </si>
   <si>
-    <t>MR THOUVENEL</t>
+    <t>MRS PAVLIDOU</t>
   </si>
   <si>
     <t>P1/S1SCHDEA</t>
   </si>
   <si>
     <t>B117</t>
-  </si>
-  <si>
-    <t>MRS PAVLIDOU</t>
   </si>
   <si>
     <t>P2/S1SCHDEA</t>
@@ -1040,10 +1037,10 @@
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>60</v>
@@ -1053,10 +1050,10 @@
       <c r="A21" s="3"/>
       <c r="B21" s="4"/>
       <c r="C21" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>64</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>60</v>
@@ -1064,16 +1061,16 @@
     </row>
     <row r="22" spans="1:5" ht="18">
       <c r="A22" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C22" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" s="5" t="s">
         <v>66</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>67</v>
       </c>
       <c r="E22" s="5"/>
     </row>
@@ -1085,18 +1082,18 @@
         <v>55</v>
       </c>
       <c r="C23" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>69</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18">
       <c r="A24" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>55</v>
@@ -1109,10 +1106,10 @@
     </row>
     <row r="25" spans="1:5" ht="18">
       <c r="A25" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>73</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
MAJ absences 2026-06-18 09:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10880" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFED1F84-82FD-4C60-81A8-11D15608395C}"/>
+  <xr:revisionPtr revIDLastSave="10881" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20E104A7-EE8D-4919-A168-2E3860929033}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
   <si>
     <t>NOMS</t>
   </si>
@@ -90,157 +90,160 @@
     <t>C107</t>
   </si>
   <si>
+    <t>MR CASTANET</t>
+  </si>
+  <si>
+    <t>P4/S1L2-DEB</t>
+  </si>
+  <si>
+    <t>MRS LÜDERS</t>
+  </si>
+  <si>
+    <t>P8/S2L3-DEB</t>
+  </si>
+  <si>
+    <t>B004</t>
+  </si>
+  <si>
+    <t>MRS KRALJIC</t>
+  </si>
+  <si>
+    <t>MRS RAYMONDAUD</t>
+  </si>
+  <si>
+    <t>P1/S4L3-FRA</t>
+  </si>
+  <si>
+    <t>B211</t>
+  </si>
+  <si>
+    <t>MRS NOBIS</t>
+  </si>
+  <si>
+    <t>P2/S3L2-FRC</t>
+  </si>
+  <si>
+    <t>B106</t>
+  </si>
+  <si>
+    <t>MRS DESROSIERS</t>
+  </si>
+  <si>
+    <t>P3/S1L2-FRB</t>
+  </si>
+  <si>
+    <t>MRS DI SALVATORE</t>
+  </si>
+  <si>
+    <t>P4/S1L2-FRB</t>
+  </si>
+  <si>
+    <t>MRS GROBER</t>
+  </si>
+  <si>
+    <t>ONLY P2 TO P8</t>
+  </si>
+  <si>
+    <t>MRS POTIN</t>
+  </si>
+  <si>
+    <t>P3/S1L2-FRA</t>
+  </si>
+  <si>
+    <t>D106</t>
+  </si>
+  <si>
+    <t>MR HADJI</t>
+  </si>
+  <si>
+    <t>P4/S1L2-FRA</t>
+  </si>
+  <si>
+    <t>MR KUPPER</t>
+  </si>
+  <si>
+    <t>P5/S3LATDEA</t>
+  </si>
+  <si>
+    <t>MR ROLL</t>
+  </si>
+  <si>
+    <t>P8/S2L3-FRA</t>
+  </si>
+  <si>
+    <t>D105</t>
+  </si>
+  <si>
+    <t>MRS PIERSON</t>
+  </si>
+  <si>
+    <t>MRS GRIRA</t>
+  </si>
+  <si>
+    <t>P5/S1L1-FRC</t>
+  </si>
+  <si>
+    <t>C202</t>
+  </si>
+  <si>
+    <t>MRS SADELER</t>
+  </si>
+  <si>
+    <t>P8/S4LATFRA</t>
+  </si>
+  <si>
+    <t>MR BOTH</t>
+  </si>
+  <si>
+    <t>MR BAZIN</t>
+  </si>
+  <si>
+    <t>P2/S4L1-ROA</t>
+  </si>
+  <si>
+    <t>B210</t>
+  </si>
+  <si>
+    <t>MRS OSKARSDOTTIR</t>
+  </si>
+  <si>
+    <t>18/06</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>MR PRIESS</t>
+  </si>
+  <si>
+    <t>MRS PAVLIDOU</t>
+  </si>
+  <si>
+    <t>P1/S1SCHDEA</t>
+  </si>
+  <si>
+    <t>B117</t>
+  </si>
+  <si>
+    <t>P2/S1SCHDEA</t>
+  </si>
+  <si>
+    <t>MRS WUTTKE</t>
+  </si>
+  <si>
+    <t>P3/S4HISDEA</t>
+  </si>
+  <si>
+    <t>MRS COSTESCU</t>
+  </si>
+  <si>
+    <t>GO TO LIBRARY</t>
+  </si>
+  <si>
+    <t>P5/S1L1ROA</t>
+  </si>
+  <si>
     <t>MR KARAGIANNIS</t>
-  </si>
-  <si>
-    <t>P4/S1L2-DEB</t>
-  </si>
-  <si>
-    <t>MRS LÜDERS</t>
-  </si>
-  <si>
-    <t>P8/S2L3-DEB</t>
-  </si>
-  <si>
-    <t>B004</t>
-  </si>
-  <si>
-    <t>MRS KRALJIC</t>
-  </si>
-  <si>
-    <t>MRS RAYMONDAUD</t>
-  </si>
-  <si>
-    <t>P1/S4L3-FRA</t>
-  </si>
-  <si>
-    <t>B211</t>
-  </si>
-  <si>
-    <t>MRS NOBIS</t>
-  </si>
-  <si>
-    <t>P2/S3L2-FRC</t>
-  </si>
-  <si>
-    <t>B106</t>
-  </si>
-  <si>
-    <t>MRS DESROSIERS</t>
-  </si>
-  <si>
-    <t>P3/S1L2-FRB</t>
-  </si>
-  <si>
-    <t>MRS DI SALVATORE</t>
-  </si>
-  <si>
-    <t>P4/S1L2-FRB</t>
-  </si>
-  <si>
-    <t>MRS GROBER</t>
-  </si>
-  <si>
-    <t>ONLY P2 TO P8</t>
-  </si>
-  <si>
-    <t>MRS POTIN</t>
-  </si>
-  <si>
-    <t>P3/S1L2-FRA</t>
-  </si>
-  <si>
-    <t>D106</t>
-  </si>
-  <si>
-    <t>MR HADJI</t>
-  </si>
-  <si>
-    <t>P4/S1L2-FRA</t>
-  </si>
-  <si>
-    <t>MR KUPPER</t>
-  </si>
-  <si>
-    <t>P5/S3LATDEA</t>
-  </si>
-  <si>
-    <t>MR ROLL</t>
-  </si>
-  <si>
-    <t>P8/S2L3-FRA</t>
-  </si>
-  <si>
-    <t>D105</t>
-  </si>
-  <si>
-    <t>MRS PIERSON</t>
-  </si>
-  <si>
-    <t>MRS GRIRA</t>
-  </si>
-  <si>
-    <t>P5/S1L1-FRC</t>
-  </si>
-  <si>
-    <t>C202</t>
-  </si>
-  <si>
-    <t>MRS SADELER</t>
-  </si>
-  <si>
-    <t>P8/S4LATFRA</t>
-  </si>
-  <si>
-    <t>MR BOTH</t>
-  </si>
-  <si>
-    <t>MR BAZIN</t>
-  </si>
-  <si>
-    <t>P2/S4L1-ROA</t>
-  </si>
-  <si>
-    <t>B210</t>
-  </si>
-  <si>
-    <t>MRS OSKARSDOTTIR</t>
-  </si>
-  <si>
-    <t>18/06</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>MR PRIESS</t>
-  </si>
-  <si>
-    <t>MRS PAVLIDOU</t>
-  </si>
-  <si>
-    <t>P1/S1SCHDEA</t>
-  </si>
-  <si>
-    <t>B117</t>
-  </si>
-  <si>
-    <t>P2/S1SCHDEA</t>
-  </si>
-  <si>
-    <t>MRS WUTTKE</t>
-  </si>
-  <si>
-    <t>P3/S4HISDEA</t>
-  </si>
-  <si>
-    <t>MRS COSTESCU</t>
-  </si>
-  <si>
-    <t>GO TO LIBRARY</t>
-  </si>
-  <si>
-    <t>P5/S1L1ROA</t>
   </si>
   <si>
     <t>MRS TOURA</t>
@@ -1076,24 +1079,24 @@
     </row>
     <row r="23" spans="1:5" ht="18">
       <c r="A23" s="3" t="s">
-        <v>16</v>
+        <v>67</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="18">
       <c r="A24" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>55</v>
@@ -1106,10 +1109,10 @@
     </row>
     <row r="25" spans="1:5" ht="18">
       <c r="A25" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>56</v>
@@ -1125,12 +1128,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1432,22 +1441,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1455,5 +1458,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-18 09:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10881" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20E104A7-EE8D-4919-A168-2E3860929033}"/>
+  <xr:revisionPtr revIDLastSave="10882" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D26BEA3-15A9-4F61-8CFB-1AFF80FB30C6}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
   <si>
     <t>NOMS</t>
   </si>
@@ -226,12 +226,6 @@
   </si>
   <si>
     <t>P2/S1SCHDEA</t>
-  </si>
-  <si>
-    <t>MRS WUTTKE</t>
-  </si>
-  <si>
-    <t>P3/S4HISDEA</t>
   </si>
   <si>
     <t>MRS COSTESCU</t>
@@ -742,7 +736,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -1050,75 +1044,62 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="3"/>
-      <c r="B21" s="4"/>
+      <c r="A21" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="C21" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>60</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="E21" s="5"/>
     </row>
     <row r="22" spans="1:5" ht="18">
       <c r="A22" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B22" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E22" s="5"/>
+        <v>67</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="23" spans="1:5" ht="18">
       <c r="A23" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>55</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>70</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
     </row>
     <row r="24" spans="1:5" ht="18">
       <c r="A24" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>71</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>56</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5" ht="18">
-      <c r="A25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1128,18 +1109,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1441,16 +1416,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1458,5 +1439,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-18 11:45
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10882" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D26BEA3-15A9-4F61-8CFB-1AFF80FB30C6}"/>
+  <xr:revisionPtr revIDLastSave="10886" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FE2915A-3737-43B9-B9DD-EE8381F1A4D6}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
   <si>
     <t>NOMS</t>
   </si>
@@ -256,6 +256,9 @@
   </si>
   <si>
     <t>ONLY P1</t>
+  </si>
+  <si>
+    <t>MRS DE PAUW</t>
   </si>
 </sst>
 </file>
@@ -736,7 +739,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U25"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -1101,6 +1104,19 @@
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
     </row>
+    <row r="25" spans="1:5" ht="18">
+      <c r="A25" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1109,12 +1125,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1416,22 +1438,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1439,5 +1455,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-18 16:35
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10886" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FE2915A-3737-43B9-B9DD-EE8381F1A4D6}"/>
+  <xr:revisionPtr revIDLastSave="10889" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{457F73A4-349D-4DF4-AA1F-58F6782AE9D6}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,205 +60,103 @@
     <t>MRS VEHLING</t>
   </si>
   <si>
-    <t>18/02</t>
-  </si>
-  <si>
-    <t>MRS NECHITA</t>
-  </si>
-  <si>
-    <t>P1/S3SCHDEA</t>
+    <t>19/06</t>
+  </si>
+  <si>
+    <t>MR GUILLOT</t>
+  </si>
+  <si>
+    <t>P3/S1SCHENC</t>
+  </si>
+  <si>
+    <t>B216</t>
+  </si>
+  <si>
+    <t>MRS CASTELLO</t>
+  </si>
+  <si>
+    <t>P5/S3SCHDEA</t>
   </si>
   <si>
     <t>B017</t>
   </si>
   <si>
-    <t>MRS DEMARTINI</t>
-  </si>
-  <si>
-    <t>P2/S1SCHENC</t>
-  </si>
-  <si>
-    <t>B216</t>
-  </si>
-  <si>
-    <t>MR ZULU</t>
-  </si>
-  <si>
-    <t>P3/S1L2-DEB</t>
+    <t>MR CHEILAS</t>
+  </si>
+  <si>
+    <t>P7/S3L3-DEA</t>
   </si>
   <si>
     <t>C107</t>
   </si>
   <si>
-    <t>MR CASTANET</t>
-  </si>
-  <si>
-    <t>P4/S1L2-DEB</t>
-  </si>
-  <si>
-    <t>MRS LÜDERS</t>
-  </si>
-  <si>
-    <t>P8/S2L3-DEB</t>
-  </si>
-  <si>
-    <t>B004</t>
+    <t>MRS PORTOGHESE</t>
+  </si>
+  <si>
+    <t>P8/S3L3-DEA</t>
   </si>
   <si>
     <t>MRS KRALJIC</t>
   </si>
   <si>
-    <t>MRS RAYMONDAUD</t>
-  </si>
-  <si>
-    <t>P1/S4L3-FRA</t>
-  </si>
-  <si>
-    <t>B211</t>
-  </si>
-  <si>
-    <t>MRS NOBIS</t>
-  </si>
-  <si>
-    <t>P2/S3L2-FRC</t>
-  </si>
-  <si>
-    <t>B106</t>
-  </si>
-  <si>
-    <t>MRS DESROSIERS</t>
-  </si>
-  <si>
-    <t>P3/S1L2-FRB</t>
-  </si>
-  <si>
-    <t>MRS DI SALVATORE</t>
-  </si>
-  <si>
-    <t>P4/S1L2-FRB</t>
-  </si>
-  <si>
-    <t>MRS GROBER</t>
-  </si>
-  <si>
-    <t>ONLY P2 TO P8</t>
-  </si>
-  <si>
-    <t>MRS POTIN</t>
-  </si>
-  <si>
-    <t>P3/S1L2-FRA</t>
-  </si>
-  <si>
-    <t>D106</t>
-  </si>
-  <si>
-    <t>MR HADJI</t>
-  </si>
-  <si>
-    <t>P4/S1L2-FRA</t>
-  </si>
-  <si>
-    <t>MR KUPPER</t>
-  </si>
-  <si>
-    <t>P5/S3LATDEA</t>
-  </si>
-  <si>
-    <t>MR ROLL</t>
-  </si>
-  <si>
-    <t>P8/S2L3-FRA</t>
-  </si>
-  <si>
-    <t>D105</t>
-  </si>
-  <si>
-    <t>MRS PIERSON</t>
-  </si>
-  <si>
-    <t>MRS GRIRA</t>
-  </si>
-  <si>
-    <t>P5/S1L1-FRC</t>
-  </si>
-  <si>
-    <t>C202</t>
-  </si>
-  <si>
-    <t>MRS SADELER</t>
-  </si>
-  <si>
-    <t>P8/S4LATFRA</t>
-  </si>
-  <si>
-    <t>MR BOTH</t>
-  </si>
-  <si>
-    <t>MR BAZIN</t>
-  </si>
-  <si>
-    <t>P2/S4L1-ROA</t>
-  </si>
-  <si>
-    <t>B210</t>
-  </si>
-  <si>
-    <t>MRS OSKARSDOTTIR</t>
-  </si>
-  <si>
-    <t>18/06</t>
-  </si>
-  <si>
     <t>*</t>
   </si>
   <si>
-    <t>MR PRIESS</t>
-  </si>
-  <si>
-    <t>MRS PAVLIDOU</t>
-  </si>
-  <si>
-    <t>P1/S1SCHDEA</t>
-  </si>
-  <si>
-    <t>B117</t>
-  </si>
-  <si>
-    <t>P2/S1SCHDEA</t>
-  </si>
-  <si>
-    <t>MRS COSTESCU</t>
+    <t>MR KARAGIANNIDIS</t>
+  </si>
+  <si>
+    <t>ONLY P6 TO P9</t>
+  </si>
+  <si>
+    <t>MR TZANOUKAKIS</t>
+  </si>
+  <si>
+    <t>ONLY P2</t>
+  </si>
+  <si>
+    <t>MRS MONTEIRO</t>
+  </si>
+  <si>
+    <t>P2/S1SCIENC</t>
+  </si>
+  <si>
+    <t>D209</t>
+  </si>
+  <si>
+    <t>MR BJERREGAARD</t>
   </si>
   <si>
     <t>GO TO LIBRARY</t>
   </si>
   <si>
-    <t>P5/S1L1ROA</t>
-  </si>
-  <si>
-    <t>MR KARAGIANNIS</t>
-  </si>
-  <si>
-    <t>MRS TOURA</t>
-  </si>
-  <si>
-    <t>P3/S2SCIELA</t>
-  </si>
-  <si>
-    <t>D210</t>
-  </si>
-  <si>
-    <t>MRS PETROULI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MR GILLIG </t>
-  </si>
-  <si>
-    <t>ONLY P1</t>
-  </si>
-  <si>
-    <t>MRS DE PAUW</t>
+    <t>P1/S4MA6DAA</t>
+  </si>
+  <si>
+    <t>C208</t>
+  </si>
+  <si>
+    <t>P2/S4MA6DAA</t>
+  </si>
+  <si>
+    <t>P3/S3MATDAA</t>
+  </si>
+  <si>
+    <t>D202</t>
+  </si>
+  <si>
+    <t>P4/S3MATDAA</t>
+  </si>
+  <si>
+    <t>P8/S2MORDAA</t>
+  </si>
+  <si>
+    <t>C203</t>
+  </si>
+  <si>
+    <t>MRS XEROU</t>
+  </si>
+  <si>
+    <t>MRS GALEZIOK</t>
   </si>
 </sst>
 </file>
@@ -739,7 +637,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -832,51 +730,55 @@
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
+      <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C6" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>20</v>
-      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+    </row>
+    <row r="8" spans="1:12" ht="18">
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="18">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
       <c r="C9" s="10" t="s">
         <v>28</v>
       </c>
@@ -884,238 +786,100 @@
         <v>29</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>31</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>33</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
       <c r="C12" s="10" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="10" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
+      <c r="A14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C14" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>43</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>47</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3"/>
       <c r="B16" s="4"/>
-      <c r="C16" s="10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>47</v>
-      </c>
+      <c r="C16" s="10"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
     </row>
     <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" spans="1:5" ht="18">
-      <c r="A19" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" ht="18">
-      <c r="A20" s="3"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" ht="18">
-      <c r="A21" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E21" s="5"/>
-    </row>
-    <row r="22" spans="1:5" ht="18">
-      <c r="A22" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="18">
-      <c r="A23" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-    </row>
-    <row r="24" spans="1:5" ht="18">
-      <c r="A24" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5" ht="18">
-      <c r="A25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -1125,18 +889,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1438,16 +1196,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1455,5 +1219,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-19 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10889" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{457F73A4-349D-4DF4-AA1F-58F6782AE9D6}"/>
+  <xr:revisionPtr revIDLastSave="10899" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6113732B-1514-4A9D-BEE4-69B41710DA5D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="toShow">Feuil1!$A:$E</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
-    <definedName name="toShow">Feuil1!$A:$E</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
   <si>
     <t>NOMS</t>
   </si>
@@ -157,6 +157,24 @@
   </si>
   <si>
     <t>MRS GALEZIOK</t>
+  </si>
+  <si>
+    <t>MRS GESTHUISEN</t>
+  </si>
+  <si>
+    <t>MRS FORÊT</t>
+  </si>
+  <si>
+    <t>ONLY P3</t>
+  </si>
+  <si>
+    <t>MRS ORMASTI</t>
+  </si>
+  <si>
+    <t>P3/S2MORFRC</t>
+  </si>
+  <si>
+    <t>B206</t>
   </si>
 </sst>
 </file>
@@ -637,7 +655,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -868,18 +886,41 @@
       <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="10"/>
+      <c r="A16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>19</v>
+      </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
     </row>
     <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="A17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -889,15 +930,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1195,6 +1227,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1211,11 +1252,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-19 11:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10899" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6113732B-1514-4A9D-BEE4-69B41710DA5D}"/>
+  <xr:revisionPtr revIDLastSave="10900" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{835A7F04-156A-495E-AE9A-FFA887560729}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,8 +16,8 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
     <definedName name="toShow">Feuil1!$A:$E</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -90,7 +90,7 @@
     <t>C107</t>
   </si>
   <si>
-    <t>MRS PORTOGHESE</t>
+    <t>MR KLOPP</t>
   </si>
   <si>
     <t>P8/S3L3-DEA</t>
@@ -930,6 +930,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1227,32 +1251,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1260,5 +1260,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-19 11:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10900" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{835A7F04-156A-495E-AE9A-FFA887560729}"/>
+  <xr:revisionPtr revIDLastSave="10901" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0892D139-4357-4074-B8C0-ECF7EBD22CE3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -90,7 +90,7 @@
     <t>C107</t>
   </si>
   <si>
-    <t>MR KLOPP</t>
+    <t>MRS MYSIRLAKI</t>
   </si>
   <si>
     <t>P8/S3L3-DEA</t>
@@ -945,15 +945,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1251,14 +1242,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-19 16:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10901" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0892D139-4357-4074-B8C0-ECF7EBD22CE3}"/>
+  <xr:revisionPtr revIDLastSave="10904" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E627532-A52A-4538-873C-EE3D71922E6D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,43 +57,46 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MRS VEHLING</t>
-  </si>
-  <si>
-    <t>19/06</t>
-  </si>
-  <si>
-    <t>MR GUILLOT</t>
-  </si>
-  <si>
-    <t>P3/S1SCHENC</t>
-  </si>
-  <si>
-    <t>B216</t>
-  </si>
-  <si>
-    <t>MRS CASTELLO</t>
-  </si>
-  <si>
-    <t>P5/S3SCHDEA</t>
-  </si>
-  <si>
-    <t>B017</t>
-  </si>
-  <si>
-    <t>MR CHEILAS</t>
-  </si>
-  <si>
-    <t>P7/S3L3-DEA</t>
-  </si>
-  <si>
-    <t>C107</t>
-  </si>
-  <si>
-    <t>MRS MYSIRLAKI</t>
-  </si>
-  <si>
-    <t>P8/S3L3-DEA</t>
+    <t>MRS GROBER</t>
+  </si>
+  <si>
+    <t>22/06</t>
+  </si>
+  <si>
+    <t>MRS TOPAL</t>
+  </si>
+  <si>
+    <t>P1/S1L2-FRA</t>
+  </si>
+  <si>
+    <t>D106</t>
+  </si>
+  <si>
+    <t>MR ZAHARIA</t>
+  </si>
+  <si>
+    <t>P2/S2L3-FRA</t>
+  </si>
+  <si>
+    <t>D105</t>
+  </si>
+  <si>
+    <t>MRS ALBERICI</t>
+  </si>
+  <si>
+    <t>P4/S2MORDEA</t>
+  </si>
+  <si>
+    <t>MRS GESTHUISEN</t>
+  </si>
+  <si>
+    <t>P7/S3LATDEA</t>
+  </si>
+  <si>
+    <t>MRS PIERSON</t>
+  </si>
+  <si>
+    <t>P8/S2LATDEA</t>
   </si>
   <si>
     <t>MRS KRALJIC</t>
@@ -102,79 +105,13 @@
     <t>*</t>
   </si>
   <si>
-    <t>MR KARAGIANNIDIS</t>
-  </si>
-  <si>
-    <t>ONLY P6 TO P9</t>
-  </si>
-  <si>
-    <t>MR TZANOUKAKIS</t>
-  </si>
-  <si>
-    <t>ONLY P2</t>
-  </si>
-  <si>
-    <t>MRS MONTEIRO</t>
-  </si>
-  <si>
-    <t>P2/S1SCIENC</t>
-  </si>
-  <si>
-    <t>D209</t>
-  </si>
-  <si>
-    <t>MR BJERREGAARD</t>
-  </si>
-  <si>
-    <t>GO TO LIBRARY</t>
-  </si>
-  <si>
-    <t>P1/S4MA6DAA</t>
-  </si>
-  <si>
-    <t>C208</t>
-  </si>
-  <si>
-    <t>P2/S4MA6DAA</t>
-  </si>
-  <si>
-    <t>P3/S3MATDAA</t>
-  </si>
-  <si>
-    <t>D202</t>
-  </si>
-  <si>
-    <t>P4/S3MATDAA</t>
-  </si>
-  <si>
-    <t>P8/S2MORDAA</t>
-  </si>
-  <si>
-    <t>C203</t>
-  </si>
-  <si>
-    <t>MRS XEROU</t>
-  </si>
-  <si>
-    <t>MRS GALEZIOK</t>
-  </si>
-  <si>
-    <t>MRS GESTHUISEN</t>
-  </si>
-  <si>
-    <t>MRS FORÊT</t>
-  </si>
-  <si>
-    <t>ONLY P3</t>
-  </si>
-  <si>
-    <t>MRS ORMASTI</t>
-  </si>
-  <si>
-    <t>P3/S2MORFRC</t>
-  </si>
-  <si>
-    <t>B206</t>
+    <t>MRS DE PAUW</t>
+  </si>
+  <si>
+    <t>MR NIKITOPOULOS</t>
+  </si>
+  <si>
+    <t>MR SNAPPE</t>
   </si>
 </sst>
 </file>
@@ -655,7 +592,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -731,196 +668,93 @@
         <v>14</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="E5" s="5" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="10" t="s">
         <v>20</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>19</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>26</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>30</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
+      <c r="A10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C10" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>30</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -930,21 +764,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1242,6 +1061,21 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1252,11 +1086,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-22 08:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10904" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E627532-A52A-4538-873C-EE3D71922E6D}"/>
+  <xr:revisionPtr revIDLastSave="10917" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DA99F74-1768-49DF-A611-7BFF1CFD2058}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>NOMS</t>
   </si>
@@ -112,6 +112,18 @@
   </si>
   <si>
     <t>MR SNAPPE</t>
+  </si>
+  <si>
+    <t>MR BERNET</t>
+  </si>
+  <si>
+    <t>MR LEADER</t>
+  </si>
+  <si>
+    <t>MRS JUHASZ</t>
+  </si>
+  <si>
+    <t>MRS FAZZARI</t>
   </si>
 </sst>
 </file>
@@ -592,7 +604,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -750,11 +762,63 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="10"/>
+      <c r="A11" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>20</v>
+      </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -764,6 +828,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1061,21 +1140,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1086,11 +1150,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-22 08:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10917" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2DA99F74-1768-49DF-A611-7BFF1CFD2058}"/>
+  <xr:revisionPtr revIDLastSave="10924" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC73AA7D-D660-4DC8-803B-32B24145DC23}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>NOMS</t>
   </si>
@@ -106,6 +106,18 @@
   </si>
   <si>
     <t>MRS DE PAUW</t>
+  </si>
+  <si>
+    <t>MRS BOUZETTE</t>
+  </si>
+  <si>
+    <t>P3/S4MA4FRB</t>
+  </si>
+  <si>
+    <t>B001</t>
+  </si>
+  <si>
+    <t>P4/S4MA4FRB</t>
   </si>
   <si>
     <t>MR NIKITOPOULOS</t>
@@ -604,7 +616,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -730,27 +742,31 @@
         <v>6</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>22</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="D9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>6</v>
@@ -763,7 +779,7 @@
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>6</v>
@@ -776,7 +792,7 @@
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>6</v>
@@ -789,7 +805,7 @@
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>6</v>
@@ -802,7 +818,7 @@
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>6</v>
@@ -814,11 +830,24 @@
       <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="10"/>
+      <c r="A15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>20</v>
+      </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-06-22 08:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10924" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC73AA7D-D660-4DC8-803B-32B24145DC23}"/>
+  <xr:revisionPtr revIDLastSave="10925" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CB0C68B-8EA5-4198-B18A-F962A68B07D9}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
   <si>
     <t>NOMS</t>
   </si>
@@ -118,9 +118,6 @@
   </si>
   <si>
     <t>P4/S4MA4FRB</t>
-  </si>
-  <si>
-    <t>MR NIKITOPOULOS</t>
   </si>
   <si>
     <t>MR SNAPPE</t>
@@ -616,7 +613,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -830,24 +827,11 @@
       <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="10"/>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -857,21 +841,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1169,6 +1138,21 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1179,11 +1163,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-22 09:40
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10925" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0CB0C68B-8EA5-4198-B18A-F962A68B07D9}"/>
+  <xr:revisionPtr revIDLastSave="10926" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C915DABB-32C4-4E6D-98A7-E5873AE4ABEA}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="30">
   <si>
     <t>NOMS</t>
   </si>
@@ -115,9 +115,6 @@
   </si>
   <si>
     <t>B001</t>
-  </si>
-  <si>
-    <t>P4/S4MA4FRB</t>
   </si>
   <si>
     <t>MR SNAPPE</t>
@@ -613,7 +610,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.85546875" customWidth="1"/>
@@ -749,17 +746,17 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C9" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>24</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
@@ -814,24 +811,11 @@
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="10"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -841,6 +825,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1138,21 +1137,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1163,11 +1147,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-06-24 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10926" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C915DABB-32C4-4E6D-98A7-E5873AE4ABEA}"/>
+  <xr:revisionPtr revIDLastSave="10931" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D5D74B5-A26B-4E7D-8B8B-38205F10FBCC}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,79 +57,13 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MRS GROBER</t>
+    <t>!MERCI DE VENIR AU BUREAU A201 SI VOTRE PROFESSEUR NE SE PRESENTE PAS EN CLASSE !</t>
   </si>
   <si>
-    <t>22/06</t>
+    <t>!PLEASE COME TO ROOM A201 IF YOUR TEACHER DOESN'T SHOW UP FOR CLASS!</t>
   </si>
   <si>
-    <t>MRS TOPAL</t>
-  </si>
-  <si>
-    <t>P1/S1L2-FRA</t>
-  </si>
-  <si>
-    <t>D106</t>
-  </si>
-  <si>
-    <t>MR ZAHARIA</t>
-  </si>
-  <si>
-    <t>P2/S2L3-FRA</t>
-  </si>
-  <si>
-    <t>D105</t>
-  </si>
-  <si>
-    <t>MRS ALBERICI</t>
-  </si>
-  <si>
-    <t>P4/S2MORDEA</t>
-  </si>
-  <si>
-    <t>MRS GESTHUISEN</t>
-  </si>
-  <si>
-    <t>P7/S3LATDEA</t>
-  </si>
-  <si>
-    <t>MRS PIERSON</t>
-  </si>
-  <si>
-    <t>P8/S2LATDEA</t>
-  </si>
-  <si>
-    <t>MRS KRALJIC</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>MRS DE PAUW</t>
-  </si>
-  <si>
-    <t>MRS BOUZETTE</t>
-  </si>
-  <si>
-    <t>P3/S4MA4FRB</t>
-  </si>
-  <si>
-    <t>B001</t>
-  </si>
-  <si>
-    <t>MR SNAPPE</t>
-  </si>
-  <si>
-    <t>MR BERNET</t>
-  </si>
-  <si>
-    <t>MR LEADER</t>
-  </si>
-  <si>
-    <t>MRS JUHASZ</t>
-  </si>
-  <si>
-    <t>MRS FAZZARI</t>
+    <t>!BITTE KOMMT ZUM BÜRO A201, WENN EUER LEHRER NICHT ZUM UNTERRICHT ERSCHEINT!</t>
   </si>
 </sst>
 </file>
@@ -646,167 +580,93 @@
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
     </row>
-    <row r="2" spans="1:12" ht="18">
+    <row r="2" spans="1:12" ht="72">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="4"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+    </row>
+    <row r="3" spans="1:12" ht="72">
+      <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+    </row>
+    <row r="4" spans="1:12" ht="72">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="18">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" ht="18">
-      <c r="A4" s="3"/>
       <c r="B4" s="4"/>
-      <c r="C4" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
-      <c r="C5" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:12" ht="18">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
-      <c r="C6" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="C6" s="10"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="10"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="10"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="10"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="10"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>20</v>
-      </c>
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="10"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
     </row>
@@ -825,18 +685,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1138,16 +992,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1155,5 +1015,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-24 08:40
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10931" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D5D74B5-A26B-4E7D-8B8B-38205F10FBCC}"/>
+  <xr:revisionPtr revIDLastSave="10934" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE4C0CCA-6693-48DF-805D-D1216A55852B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -112,7 +112,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -185,11 +185,85 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -220,6 +294,24 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -580,30 +672,30 @@
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
     </row>
-    <row r="2" spans="1:12" ht="72">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:12" ht="72" customHeight="1">
+      <c r="A2" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="10"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="13"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" spans="1:12" ht="72">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:12" ht="72" customHeight="1">
+      <c r="A3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="10"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="16"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:12" ht="72">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:12" ht="72" customHeight="1">
+      <c r="A4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="10"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="16"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
     </row>
@@ -678,6 +770,11 @@
       <c r="E14" s="5"/>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+  </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
@@ -694,6 +791,21 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -991,29 +1103,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-06-24 08:45
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10934" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE4C0CCA-6693-48DF-805D-D1216A55852B}"/>
+  <xr:revisionPtr revIDLastSave="10947" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC648DA9-9ADB-4544-8205-5D32416DDC3C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -112,7 +112,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -199,30 +199,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -237,25 +213,64 @@
     </border>
     <border>
       <left/>
+      <right style="double">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
       <right/>
       <top style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
       </top>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -263,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -283,9 +298,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -296,22 +308,28 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,7 +657,7 @@
   <dimension ref="A1:U14"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="40.85546875" customWidth="1"/>
+    <col min="1" max="1" width="90.28515625" customWidth="1"/>
     <col min="2" max="2" width="33.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="37.7109375" customWidth="1"/>
     <col min="4" max="4" width="30.28515625" customWidth="1"/>
@@ -652,16 +670,16 @@
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="2"/>
@@ -673,108 +691,103 @@
       <c r="L1" s="2"/>
     </row>
     <row r="2" spans="1:12" ht="72" customHeight="1">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="15"/>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:12" ht="72" customHeight="1">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="15"/>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
     <row r="4" spans="1:12" ht="72" customHeight="1">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="15"/>
-      <c r="C4" s="16"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="14"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
-      <c r="C5" s="10"/>
+      <c r="C5" s="9"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:12" ht="18">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
-      <c r="C6" s="10"/>
+      <c r="C6" s="9"/>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3"/>
       <c r="B7" s="4"/>
-      <c r="C7" s="10"/>
+      <c r="C7" s="9"/>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
-      <c r="C8" s="10"/>
+      <c r="C8" s="9"/>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
-      <c r="C9" s="10"/>
+      <c r="C9" s="9"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
-      <c r="C10" s="10"/>
+      <c r="C10" s="9"/>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
-      <c r="C11" s="10"/>
+      <c r="C11" s="9"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>
       <c r="B12" s="4"/>
-      <c r="C12" s="10"/>
+      <c r="C12" s="9"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="10"/>
+      <c r="C13" s="9"/>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="10"/>
+      <c r="C14" s="9"/>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-  </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
MAJ absences 2026-09-01 15:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10947" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC648DA9-9ADB-4544-8205-5D32416DDC3C}"/>
+  <xr:revisionPtr revIDLastSave="10956" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE13A942-8E17-4E5B-850F-B11C8BBE1DF2}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,20 +57,47 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>!MERCI DE VENIR AU BUREAU A201 SI VOTRE PROFESSEUR NE SE PRESENTE PAS EN CLASSE !</t>
-  </si>
-  <si>
-    <t>!PLEASE COME TO ROOM A201 IF YOUR TEACHER DOESN'T SHOW UP FOR CLASS!</t>
-  </si>
-  <si>
-    <t>!BITTE KOMMT ZUM BÜRO A201, WENN EUER LEHRER NICHT ZUM UNTERRICHT ERSCHEINT!</t>
+    <t>MR HEDBERG</t>
+  </si>
+  <si>
+    <t>02/09</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>MRS PORTOGHESE</t>
+  </si>
+  <si>
+    <t>MRS ANDERSSON</t>
+  </si>
+  <si>
+    <t>ONLY P3</t>
+  </si>
+  <si>
+    <t>MRS BOUZETTE</t>
+  </si>
+  <si>
+    <t>ONLY P3 TO P9</t>
+  </si>
+  <si>
+    <t>MR BOTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONLY P3 </t>
+  </si>
+  <si>
+    <t>MR COUCHE</t>
+  </si>
+  <si>
+    <t>MR GRIRA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,13 +106,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Verdana"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <u/>
       <sz val="14"/>
       <color theme="1"/>
       <name val="Verdana"/>
@@ -112,7 +132,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -185,100 +205,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="double">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -286,13 +217,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -304,32 +235,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -654,10 +561,10 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="90.28515625" customWidth="1"/>
+    <col min="1" max="1" width="40.5703125" customWidth="1"/>
     <col min="2" max="2" width="33.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="37.7109375" customWidth="1"/>
     <col min="4" max="4" width="30.28515625" customWidth="1"/>
@@ -670,10 +577,10 @@
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
@@ -690,58 +597,94 @@
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
     </row>
-    <row r="2" spans="1:12" ht="72" customHeight="1">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:12" ht="21" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="16"/>
-      <c r="C2" s="15"/>
+      <c r="B2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" spans="1:12" ht="72" customHeight="1">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:12" ht="18.75" customHeight="1">
+      <c r="A3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="15"/>
+      <c r="C3" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:12" ht="72" customHeight="1">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:12" ht="20.25" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="14"/>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:12" ht="18">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="9"/>
+      <c r="A5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
     <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="9"/>
+      <c r="A6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="9"/>
+      <c r="A7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="9"/>
+      <c r="A8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
@@ -752,43 +695,8 @@
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-    </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
 </worksheet>
@@ -804,21 +712,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1116,14 +1009,29 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-01 16:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10956" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE13A942-8E17-4E5B-850F-B11C8BBE1DF2}"/>
+  <xr:revisionPtr revIDLastSave="10958" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A055B63F-42C7-4363-A788-99F8D1E37499}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -565,7 +565,7 @@
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
-    <col min="2" max="2" width="33.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="37.7109375" customWidth="1"/>
     <col min="4" max="4" width="30.28515625" customWidth="1"/>
     <col min="5" max="5" width="29" customWidth="1"/>

</xml_diff>

<commit_message>
MAJ absences 2026-09-02 10:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10958" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A055B63F-42C7-4363-A788-99F8D1E37499}"/>
+  <xr:revisionPtr revIDLastSave="10972" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E76D0BD4-B473-4AC2-BBD8-04C0C86A975B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$6</definedName>
     <definedName name="toShow">Feuil1!$A:$E</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
   <si>
     <t>NOMS</t>
   </si>
@@ -67,6 +67,21 @@
   </si>
   <si>
     <t>MRS PORTOGHESE</t>
+  </si>
+  <si>
+    <t>MR ORIOLO</t>
+  </si>
+  <si>
+    <t>P6/S7L3ITA</t>
+  </si>
+  <si>
+    <t>D114</t>
+  </si>
+  <si>
+    <t>P7/S7L3ITA</t>
+  </si>
+  <si>
+    <t>P8/S3S1ITB</t>
   </si>
   <si>
     <t>MRS ANDERSSON</t>
@@ -561,7 +576,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -618,43 +633,47 @@
         <v>6</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:12" ht="20.25" customHeight="1">
-      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="E3" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="18.75" customHeight="1">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-    </row>
-    <row r="5" spans="1:12" ht="18">
-      <c r="A5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>12</v>
-      </c>
+    </row>
+    <row r="5" spans="1:12" ht="18.75" customHeight="1">
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-    </row>
-    <row r="6" spans="1:12" ht="18">
+        <v>9</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="20.25" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>7</v>
@@ -664,10 +683,10 @@
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>7</v>
@@ -677,10 +696,10 @@
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>7</v>
@@ -689,11 +708,44 @@
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="9"/>
+      <c r="A9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
+    </row>
+    <row r="10" spans="1:12" ht="18">
+      <c r="A10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -703,15 +755,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1009,6 +1052,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1025,11 +1077,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-02 16:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10972" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E76D0BD4-B473-4AC2-BBD8-04C0C86A975B}"/>
+  <xr:revisionPtr revIDLastSave="10978" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C76A28A-DEDB-4298-BF07-D8A57E9BD1E3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,52 +60,79 @@
     <t>MR HEDBERG</t>
   </si>
   <si>
-    <t>02/09</t>
+    <t>03/09</t>
+  </si>
+  <si>
+    <t>MRS KASTANIDOU</t>
+  </si>
+  <si>
+    <t>P2/S1L2-ENA</t>
+  </si>
+  <si>
+    <t>C209</t>
+  </si>
+  <si>
+    <t>MRS PORTOGHESE</t>
+  </si>
+  <si>
+    <t>MRS GIORGERINI</t>
+  </si>
+  <si>
+    <t>P3/S7L4-ITA</t>
+  </si>
+  <si>
+    <t>B114</t>
+  </si>
+  <si>
+    <t>MRS BENETTI</t>
+  </si>
+  <si>
+    <t>P4/S7L4-ITA</t>
+  </si>
+  <si>
+    <t>MRS ROMANO</t>
+  </si>
+  <si>
+    <t>P6/S2LATITA</t>
+  </si>
+  <si>
+    <t>MR ORIOLO</t>
+  </si>
+  <si>
+    <t>P7/S7L3-ITA</t>
+  </si>
+  <si>
+    <t>P9/S4L1-ITA</t>
+  </si>
+  <si>
+    <t>MRS GRIRA</t>
+  </si>
+  <si>
+    <t>MRS BOUZETTE</t>
+  </si>
+  <si>
+    <t>P4/S2MATFRC</t>
+  </si>
+  <si>
+    <t>B214</t>
+  </si>
+  <si>
+    <t>MR ANYFANTAKIS</t>
+  </si>
+  <si>
+    <t>MRS DI SALVATORE</t>
+  </si>
+  <si>
+    <t>P4/S2RORELA</t>
+  </si>
+  <si>
+    <t>B212</t>
+  </si>
+  <si>
+    <t>MR MORABITO</t>
   </si>
   <si>
     <t>*</t>
-  </si>
-  <si>
-    <t>MRS PORTOGHESE</t>
-  </si>
-  <si>
-    <t>MR ORIOLO</t>
-  </si>
-  <si>
-    <t>P6/S7L3ITA</t>
-  </si>
-  <si>
-    <t>D114</t>
-  </si>
-  <si>
-    <t>P7/S7L3ITA</t>
-  </si>
-  <si>
-    <t>P8/S3S1ITB</t>
-  </si>
-  <si>
-    <t>MRS ANDERSSON</t>
-  </si>
-  <si>
-    <t>ONLY P3</t>
-  </si>
-  <si>
-    <t>MRS BOUZETTE</t>
-  </si>
-  <si>
-    <t>ONLY P3 TO P9</t>
-  </si>
-  <si>
-    <t>MR BOTH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ONLY P3 </t>
-  </si>
-  <si>
-    <t>MR COUCHE</t>
-  </si>
-  <si>
-    <t>MR GRIRA</t>
   </si>
 </sst>
 </file>
@@ -622,113 +649,125 @@
       <c r="C2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="18.75" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18.75" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="9" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
-      <c r="A6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+        <v>18</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+      <c r="D7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>22</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+        <v>26</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
@@ -755,6 +794,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1052,15 +1100,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1077,11 +1116,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-02 16:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10978" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C76A28A-DEDB-4298-BF07-D8A57E9BD1E3}"/>
+  <xr:revisionPtr revIDLastSave="10979" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3DB744F-7811-403F-9BC2-C84F16CC74D5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -108,7 +108,7 @@
     <t>MRS GRIRA</t>
   </si>
   <si>
-    <t>MRS BOUZETTE</t>
+    <t>MRS ANCEL</t>
   </si>
   <si>
     <t>P4/S2MATFRC</t>

</xml_diff>

<commit_message>
MAJ absences 2026-09-03 08:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10979" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3DB744F-7811-403F-9BC2-C84F16CC74D5}"/>
+  <xr:revisionPtr revIDLastSave="10993" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E0DF456-507C-4D4F-AD12-377F749B5205}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
   <si>
     <t>NOMS</t>
   </si>
@@ -120,19 +120,34 @@
     <t>MR ANYFANTAKIS</t>
   </si>
   <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>P4/S2RORELA</t>
+  </si>
+  <si>
+    <t>B212</t>
+  </si>
+  <si>
+    <t>MR MORABITO</t>
+  </si>
+  <si>
+    <t>MR KARAGIANNIS</t>
+  </si>
+  <si>
+    <t>MR CIUCULESCU</t>
+  </si>
+  <si>
     <t>MRS DI SALVATORE</t>
   </si>
   <si>
-    <t>P4/S2RORELA</t>
-  </si>
-  <si>
-    <t>B212</t>
-  </si>
-  <si>
-    <t>MR MORABITO</t>
-  </si>
-  <si>
-    <t>*</t>
+    <t>MRS JUHASZ</t>
+  </si>
+  <si>
+    <t>P3/S1RCAITA</t>
+  </si>
+  <si>
+    <t>B016</t>
   </si>
 </sst>
 </file>
@@ -603,7 +618,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -767,24 +782,53 @@
         <v>6</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="9"/>
+      <c r="A11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="9"/>
+      <c r="A12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>26</v>
+      </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -803,6 +847,21 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1100,29 +1159,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-03 09:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10993" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E0DF456-507C-4D4F-AD12-377F749B5205}"/>
+  <xr:revisionPtr revIDLastSave="11002" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F51C9F7D-FE4C-4B5E-B84F-B41EDCF01E2D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>NOMS</t>
   </si>
@@ -148,13 +148,28 @@
   </si>
   <si>
     <t>B016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MR HEDBERG </t>
+  </si>
+  <si>
+    <t>ONLY P7 TO P8</t>
+  </si>
+  <si>
+    <t>MR BOTH</t>
+  </si>
+  <si>
+    <t>P7/P8/S6PHENA</t>
+  </si>
+  <si>
+    <t>A202</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,6 +192,13 @@
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Verdana"/>
       <family val="2"/>
     </font>
@@ -266,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -294,6 +316,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -618,7 +652,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -830,6 +864,30 @@
         <v>35</v>
       </c>
     </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -838,30 +896,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1159,8 +1193,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1168,5 +1226,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-03 11:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11002" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F51C9F7D-FE4C-4B5E-B84F-B41EDCF01E2D}"/>
+  <xr:revisionPtr revIDLastSave="11009" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8159C7FE-9F70-463E-BB72-353D58944EEF}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
   <si>
     <t>NOMS</t>
   </si>
@@ -163,6 +163,18 @@
   </si>
   <si>
     <t>A202</t>
+  </si>
+  <si>
+    <t>ONLY P6</t>
+  </si>
+  <si>
+    <t>GO TO SSV S4 ASSEMBLY</t>
+  </si>
+  <si>
+    <t>P6</t>
+  </si>
+  <si>
+    <t>SSV</t>
   </si>
 </sst>
 </file>
@@ -881,12 +893,22 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+    <row r="15" spans="1:12" ht="36">
+      <c r="A15" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -896,6 +918,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1193,21 +1230,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1218,11 +1240,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-03 16:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11009" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8159C7FE-9F70-463E-BB72-353D58944EEF}"/>
+  <xr:revisionPtr revIDLastSave="11011" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7432442-93A6-4A66-A5BF-A8DCBB35F98A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,16 +57,49 @@
     <t>SALLES</t>
   </si>
   <si>
+    <t>MRS GRIRA</t>
+  </si>
+  <si>
+    <t>04/09</t>
+  </si>
+  <si>
+    <t>MRS ANCEL</t>
+  </si>
+  <si>
+    <t>P1/S1MATFRA</t>
+  </si>
+  <si>
+    <t>B216</t>
+  </si>
+  <si>
+    <t>MRS FAIVRE</t>
+  </si>
+  <si>
+    <t>P2/S1MATFRA</t>
+  </si>
+  <si>
+    <t>MR BERRICHI</t>
+  </si>
+  <si>
+    <t>P6/S3MATFRA</t>
+  </si>
+  <si>
+    <t>C110</t>
+  </si>
+  <si>
+    <t>MRS WUTTKE</t>
+  </si>
+  <si>
+    <t>P7/S3MATFRA</t>
+  </si>
+  <si>
     <t>MR HEDBERG</t>
   </si>
   <si>
-    <t>03/09</t>
-  </si>
-  <si>
-    <t>MRS KASTANIDOU</t>
-  </si>
-  <si>
-    <t>P2/S1L2-ENA</t>
+    <t>MR MULRENNAN</t>
+  </si>
+  <si>
+    <t>P6/S1L2-ENA</t>
   </si>
   <si>
     <t>C209</t>
@@ -75,106 +108,34 @@
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
+    <t>MRS VERZELETTI</t>
+  </si>
+  <si>
+    <t>P2/S3L1-ITB</t>
+  </si>
+  <si>
+    <t>B114</t>
+  </si>
+  <si>
     <t>MRS GIORGERINI</t>
   </si>
   <si>
-    <t>P3/S7L4-ITA</t>
-  </si>
-  <si>
-    <t>B114</t>
+    <t>P5/S7L4-ITA</t>
   </si>
   <si>
     <t>MRS BENETTI</t>
   </si>
   <si>
-    <t>P4/S7L4-ITA</t>
+    <t>P7/S1L3-ITA</t>
   </si>
   <si>
     <t>MRS ROMANO</t>
   </si>
   <si>
-    <t>P6/S2LATITA</t>
-  </si>
-  <si>
-    <t>MR ORIOLO</t>
-  </si>
-  <si>
-    <t>P7/S7L3-ITA</t>
-  </si>
-  <si>
-    <t>P9/S4L1-ITA</t>
-  </si>
-  <si>
-    <t>MRS GRIRA</t>
-  </si>
-  <si>
-    <t>MRS ANCEL</t>
-  </si>
-  <si>
-    <t>P4/S2MATFRC</t>
-  </si>
-  <si>
-    <t>B214</t>
-  </si>
-  <si>
-    <t>MR ANYFANTAKIS</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>P4/S2RORELA</t>
-  </si>
-  <si>
-    <t>B212</t>
-  </si>
-  <si>
-    <t>MR MORABITO</t>
-  </si>
-  <si>
-    <t>MR KARAGIANNIS</t>
-  </si>
-  <si>
-    <t>MR CIUCULESCU</t>
-  </si>
-  <si>
-    <t>MRS DI SALVATORE</t>
-  </si>
-  <si>
-    <t>MRS JUHASZ</t>
-  </si>
-  <si>
-    <t>P3/S1RCAITA</t>
-  </si>
-  <si>
-    <t>B016</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MR HEDBERG </t>
-  </si>
-  <si>
-    <t>ONLY P7 TO P8</t>
-  </si>
-  <si>
-    <t>MR BOTH</t>
-  </si>
-  <si>
-    <t>P7/P8/S6PHENA</t>
-  </si>
-  <si>
-    <t>A202</t>
-  </si>
-  <si>
-    <t>ONLY P6</t>
-  </si>
-  <si>
-    <t>GO TO SSV S4 ASSEMBLY</t>
-  </si>
-  <si>
-    <t>P6</t>
-  </si>
-  <si>
-    <t>SSV</t>
+    <t>P8/S4L1-ITA</t>
+  </si>
+  <si>
+    <t>P9/S3LATITA</t>
   </si>
 </sst>
 </file>
@@ -718,51 +679,51 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>12</v>
-      </c>
       <c r="E3" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="18.75" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18.75" customHeight="1">
       <c r="A5" s="3"/>
       <c r="B5" s="4"/>
       <c r="C5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="20.25" customHeight="1">
+      <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="20.25" customHeight="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
+      <c r="B6" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C6" s="9" t="s">
         <v>18</v>
       </c>
@@ -770,145 +731,105 @@
         <v>19</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C7" s="9" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="9" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
       <c r="C9" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="18">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E9" s="5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>26</v>
-      </c>
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="9"/>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>35</v>
-      </c>
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="36">
-      <c r="A15" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>44</v>
-      </c>
+      <c r="A14" s="10"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="10"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -918,18 +839,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1231,16 +1146,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1248,5 +1169,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-04 08:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11011" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7432442-93A6-4A66-A5BF-A8DCBB35F98A}"/>
+  <xr:revisionPtr revIDLastSave="11022" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{937A296A-DFE0-4F08-AFEE-25168A969252}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>NOMS</t>
   </si>
@@ -136,6 +136,24 @@
   </si>
   <si>
     <t>P9/S3LATITA</t>
+  </si>
+  <si>
+    <t>MRS DUFF</t>
+  </si>
+  <si>
+    <t>MRS COQUELIN</t>
+  </si>
+  <si>
+    <t>P7/S2SCHENC</t>
+  </si>
+  <si>
+    <t>B009</t>
+  </si>
+  <si>
+    <t>MRS VEHLING</t>
+  </si>
+  <si>
+    <t>P8/S2SCHENC</t>
   </si>
 </sst>
 </file>
@@ -804,18 +822,34 @@
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="A12" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="C13" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="10"/>
@@ -839,12 +873,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1146,22 +1186,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1169,5 +1203,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-04 08:15
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11022" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{937A296A-DFE0-4F08-AFEE-25168A969252}"/>
+  <xr:revisionPtr revIDLastSave="11027" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7372CEFD-976E-42CD-A1D4-DAB596D3E422}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
   <si>
     <t>NOMS</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>P8/S2SCHENC</t>
+  </si>
+  <si>
+    <t>MR CHAVET</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -852,9 +858,15 @@
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="12"/>
+      <c r="A14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
     </row>

</xml_diff>

<commit_message>
MAJ absences 2026-09-04 08:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11027" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7372CEFD-976E-42CD-A1D4-DAB596D3E422}"/>
+  <xr:revisionPtr revIDLastSave="11029" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F84C8F6-C68C-448D-8262-7E382323DA06}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="41">
   <si>
     <t>NOMS</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t>MRS DUFF</t>
+  </si>
+  <si>
+    <t>!ONLY P7 TO P8</t>
   </si>
   <si>
     <t>MRS COQUELIN</t>
@@ -832,40 +835,40 @@
         <v>32</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>
       <c r="B13" s="4"/>
       <c r="C13" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>36</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>

</xml_diff>

<commit_message>
MAJ absences 2026-09-04 08:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11029" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F84C8F6-C68C-448D-8262-7E382323DA06}"/>
+  <xr:revisionPtr revIDLastSave="11030" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDC972B3-D777-471E-A247-269029901830}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -169,7 +169,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -201,6 +201,11 @@
       <color rgb="FFFF0000"/>
       <name val="Verdana"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Verdana"/>
     </font>
   </fonts>
   <fills count="2">
@@ -288,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -328,6 +333,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -834,7 +842,7 @@
       <c r="A12" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="14" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="9" t="s">

</xml_diff>

<commit_message>
MAJ absences 2026-09-04 16:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11030" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDC972B3-D777-471E-A247-269029901830}"/>
+  <xr:revisionPtr revIDLastSave="11033" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{592E0F65-EB0F-4941-A52B-6CD239B8A413}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,112 +57,109 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MRS GRIRA</t>
-  </si>
-  <si>
-    <t>04/09</t>
-  </si>
-  <si>
-    <t>MRS ANCEL</t>
-  </si>
-  <si>
-    <t>P1/S1MATFRA</t>
-  </si>
-  <si>
-    <t>B216</t>
-  </si>
-  <si>
-    <t>MRS FAIVRE</t>
-  </si>
-  <si>
-    <t>P2/S1MATFRA</t>
-  </si>
-  <si>
-    <t>MR BERRICHI</t>
-  </si>
-  <si>
-    <t>P6/S3MATFRA</t>
-  </si>
-  <si>
-    <t>C110</t>
-  </si>
-  <si>
-    <t>MRS WUTTKE</t>
-  </si>
-  <si>
-    <t>P7/S3MATFRA</t>
+    <t>MR ANYFANTAKIS</t>
+  </si>
+  <si>
+    <t>07/09</t>
+  </si>
+  <si>
+    <t>MR ATCHADE</t>
+  </si>
+  <si>
+    <t>P3/S1RORELA</t>
+  </si>
+  <si>
+    <t>A111</t>
   </si>
   <si>
     <t>MR HEDBERG</t>
   </si>
   <si>
-    <t>MR MULRENNAN</t>
-  </si>
-  <si>
-    <t>P6/S1L2-ENA</t>
+    <t>MR LEADER</t>
+  </si>
+  <si>
+    <t>P1/S7L2-ENA</t>
   </si>
   <si>
     <t>C209</t>
   </si>
   <si>
+    <t>P2/S7L2-ENA</t>
+  </si>
+  <si>
+    <t>MRS WILES</t>
+  </si>
+  <si>
+    <t>P8/S4L3-ENB</t>
+  </si>
+  <si>
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
     <t>MRS VERZELETTI</t>
   </si>
   <si>
-    <t>P2/S3L1-ITB</t>
+    <t>P1/S1L3-ITA</t>
   </si>
   <si>
     <t>B114</t>
   </si>
   <si>
-    <t>MRS GIORGERINI</t>
-  </si>
-  <si>
-    <t>P5/S7L4-ITA</t>
-  </si>
-  <si>
     <t>MRS BENETTI</t>
   </si>
   <si>
-    <t>P7/S1L3-ITA</t>
-  </si>
-  <si>
-    <t>MRS ROMANO</t>
-  </si>
-  <si>
-    <t>P8/S4L1-ITA</t>
-  </si>
-  <si>
-    <t>P9/S3LATITA</t>
-  </si>
-  <si>
-    <t>MRS DUFF</t>
-  </si>
-  <si>
-    <t>!ONLY P7 TO P8</t>
-  </si>
-  <si>
-    <t>MRS COQUELIN</t>
-  </si>
-  <si>
-    <t>P7/S2SCHENC</t>
-  </si>
-  <si>
-    <t>B009</t>
-  </si>
-  <si>
-    <t>MRS VEHLING</t>
-  </si>
-  <si>
-    <t>P8/S2SCHENC</t>
-  </si>
-  <si>
-    <t>MR CHAVET</t>
+    <t>P5/S7L3-ITA</t>
+  </si>
+  <si>
+    <t>P9/S7L4-ITA</t>
+  </si>
+  <si>
+    <t>MRS CASTANET</t>
+  </si>
+  <si>
+    <t>MRS MAQUET</t>
+  </si>
+  <si>
+    <t>P4/S2SCIFRA</t>
+  </si>
+  <si>
+    <t>D204</t>
+  </si>
+  <si>
+    <t>MRS LUC</t>
+  </si>
+  <si>
+    <t>P7/S2SCIFRA</t>
+  </si>
+  <si>
+    <t>D209</t>
+  </si>
+  <si>
+    <t>MRS RHEINHEIMER</t>
+  </si>
+  <si>
+    <t>P8/S2SCIFRD</t>
+  </si>
+  <si>
+    <t>MRS STRAUS ZULU</t>
   </si>
   <si>
     <t>*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MRS NECHITA </t>
+  </si>
+  <si>
+    <t>MRS CONNOLLY</t>
+  </si>
+  <si>
+    <t>P1/S1L3-ENB</t>
+  </si>
+  <si>
+    <t>C001</t>
+  </si>
+  <si>
+    <t>MR PARKER</t>
   </si>
 </sst>
 </file>
@@ -204,7 +201,7 @@
     </font>
     <font>
       <sz val="14"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF000000"/>
       <name val="Verdana"/>
     </font>
   </fonts>
@@ -714,29 +711,33 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C3" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="18.75" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18.75" customHeight="1">
@@ -749,7 +750,7 @@
         <v>16</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
@@ -770,102 +771,102 @@
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="E7" s="5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3"/>
       <c r="B8" s="4"/>
       <c r="C8" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="18">
+      <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="9" t="s">
+      <c r="E9" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
       <c r="C10" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3"/>
       <c r="B11" s="4"/>
       <c r="C11" s="9" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="B13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>38</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="18">
@@ -876,7 +877,7 @@
         <v>6</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
@@ -896,18 +897,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1209,16 +1204,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1226,5 +1227,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-07 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11033" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{592E0F65-EB0F-4941-A52B-6CD239B8A413}"/>
+  <xr:revisionPtr revIDLastSave="11042" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{806740AF-EB14-46EC-91DF-B62243074B01}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
   <si>
     <t>NOMS</t>
   </si>
@@ -160,6 +160,15 @@
   </si>
   <si>
     <t>MR PARKER</t>
+  </si>
+  <si>
+    <t>MR NESTORAS</t>
+  </si>
+  <si>
+    <t>ONLY P2</t>
+  </si>
+  <si>
+    <t>MRS GROBER</t>
   </si>
 </sst>
 </file>
@@ -290,7 +299,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -317,15 +326,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -657,7 +657,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -843,7 +843,7 @@
       <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="11" t="s">
         <v>6</v>
       </c>
       <c r="C12" s="9" t="s">
@@ -879,15 +879,41 @@
       <c r="C14" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
     </row>
     <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
+      <c r="A15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -897,12 +923,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1204,22 +1236,16 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1227,5 +1253,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-07 08:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11042" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{806740AF-EB14-46EC-91DF-B62243074B01}"/>
+  <xr:revisionPtr revIDLastSave="11047" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C68BDBCC-7ADE-4690-AE33-6A3B887F5678}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
   <si>
     <t>NOMS</t>
   </si>
@@ -169,6 +169,12 @@
   </si>
   <si>
     <t>MRS GROBER</t>
+  </si>
+  <si>
+    <t>P2/S2MATENC</t>
+  </si>
+  <si>
+    <t>B015</t>
   </si>
 </sst>
 </file>
@@ -905,15 +911,19 @@
       <c r="C16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
+      <c r="D16" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="17" spans="1:5" ht="18">
       <c r="A17" s="3"/>
       <c r="B17" s="4"/>
       <c r="C17" s="9"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-09-07 08:15
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11047" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C68BDBCC-7ADE-4690-AE33-6A3B887F5678}"/>
+  <xr:revisionPtr revIDLastSave="11048" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F529D8A4-DAD1-4B58-B757-98AD796EC950}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
   <si>
     <t>NOMS</t>
   </si>
@@ -63,103 +63,106 @@
     <t>07/09</t>
   </si>
   <si>
+    <t>MR STEFANIS</t>
+  </si>
+  <si>
+    <t>P3/S1RORELA</t>
+  </si>
+  <si>
+    <t>A111</t>
+  </si>
+  <si>
+    <t>MR HEDBERG</t>
+  </si>
+  <si>
+    <t>MR LEADER</t>
+  </si>
+  <si>
+    <t>P1/S7L2-ENA</t>
+  </si>
+  <si>
+    <t>C209</t>
+  </si>
+  <si>
+    <t>P2/S7L2-ENA</t>
+  </si>
+  <si>
+    <t>MRS WILES</t>
+  </si>
+  <si>
+    <t>P8/S4L3-ENB</t>
+  </si>
+  <si>
+    <t>MRS PORTOGHESE</t>
+  </si>
+  <si>
+    <t>MRS VERZELETTI</t>
+  </si>
+  <si>
+    <t>P1/S1L3-ITA</t>
+  </si>
+  <si>
+    <t>B114</t>
+  </si>
+  <si>
+    <t>MRS BENETTI</t>
+  </si>
+  <si>
+    <t>P5/S7L3-ITA</t>
+  </si>
+  <si>
+    <t>P9/S7L4-ITA</t>
+  </si>
+  <si>
+    <t>MRS CASTANET</t>
+  </si>
+  <si>
+    <t>MRS MAQUET</t>
+  </si>
+  <si>
+    <t>P4/S2SCIFRA</t>
+  </si>
+  <si>
+    <t>D204</t>
+  </si>
+  <si>
+    <t>MRS LUC</t>
+  </si>
+  <si>
+    <t>P7/S2SCIFRA</t>
+  </si>
+  <si>
+    <t>D209</t>
+  </si>
+  <si>
+    <t>MRS RHEINHEIMER</t>
+  </si>
+  <si>
+    <t>P8/S2SCIFRD</t>
+  </si>
+  <si>
+    <t>MRS STRAUS ZULU</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MRS NECHITA </t>
+  </si>
+  <si>
+    <t>MRS CONNOLLY</t>
+  </si>
+  <si>
+    <t>P1/S1L3-ENB</t>
+  </si>
+  <si>
+    <t>C001</t>
+  </si>
+  <si>
+    <t>MR PARKER</t>
+  </si>
+  <si>
     <t>MR ATCHADE</t>
-  </si>
-  <si>
-    <t>P3/S1RORELA</t>
-  </si>
-  <si>
-    <t>A111</t>
-  </si>
-  <si>
-    <t>MR HEDBERG</t>
-  </si>
-  <si>
-    <t>MR LEADER</t>
-  </si>
-  <si>
-    <t>P1/S7L2-ENA</t>
-  </si>
-  <si>
-    <t>C209</t>
-  </si>
-  <si>
-    <t>P2/S7L2-ENA</t>
-  </si>
-  <si>
-    <t>MRS WILES</t>
-  </si>
-  <si>
-    <t>P8/S4L3-ENB</t>
-  </si>
-  <si>
-    <t>MRS PORTOGHESE</t>
-  </si>
-  <si>
-    <t>MRS VERZELETTI</t>
-  </si>
-  <si>
-    <t>P1/S1L3-ITA</t>
-  </si>
-  <si>
-    <t>B114</t>
-  </si>
-  <si>
-    <t>MRS BENETTI</t>
-  </si>
-  <si>
-    <t>P5/S7L3-ITA</t>
-  </si>
-  <si>
-    <t>P9/S7L4-ITA</t>
-  </si>
-  <si>
-    <t>MRS CASTANET</t>
-  </si>
-  <si>
-    <t>MRS MAQUET</t>
-  </si>
-  <si>
-    <t>P4/S2SCIFRA</t>
-  </si>
-  <si>
-    <t>D204</t>
-  </si>
-  <si>
-    <t>MRS LUC</t>
-  </si>
-  <si>
-    <t>P7/S2SCIFRA</t>
-  </si>
-  <si>
-    <t>D209</t>
-  </si>
-  <si>
-    <t>MRS RHEINHEIMER</t>
-  </si>
-  <si>
-    <t>P8/S2SCIFRD</t>
-  </si>
-  <si>
-    <t>MRS STRAUS ZULU</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MRS NECHITA </t>
-  </si>
-  <si>
-    <t>MRS CONNOLLY</t>
-  </si>
-  <si>
-    <t>P1/S1L3-ENB</t>
-  </si>
-  <si>
-    <t>C001</t>
-  </si>
-  <si>
-    <t>MR PARKER</t>
   </si>
   <si>
     <t>MR NESTORAS</t>
@@ -890,7 +893,7 @@
     </row>
     <row r="15" spans="1:12" ht="18">
       <c r="A15" s="3" t="s">
-        <v>7</v>
+        <v>40</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>6</v>
@@ -903,19 +906,19 @@
     </row>
     <row r="16" spans="1:12" ht="18">
       <c r="A16" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="18">

</xml_diff>

<commit_message>
MAJ absences 2026-09-07 10:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11048" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F529D8A4-DAD1-4B58-B757-98AD796EC950}"/>
+  <xr:revisionPtr revIDLastSave="11050" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C29BEAC8-F1B8-4595-8481-9AB4F92989AC}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -129,7 +129,23 @@
     <t>MRS LUC</t>
   </si>
   <si>
-    <t>P7/S2SCIFRA</t>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF000000"/>
+        <rFont val="Verdana"/>
+      </rPr>
+      <t>P7/S2SCIFR</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Verdana"/>
+      </rPr>
+      <t>D</t>
+    </r>
   </si>
   <si>
     <t>D209</t>
@@ -184,7 +200,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,6 +236,12 @@
     <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
+      <name val="Verdana"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
       <name val="Verdana"/>
     </font>
   </fonts>
@@ -308,7 +330,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -342,6 +364,9 @@
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -828,7 +853,7 @@
       <c r="C10" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="12" t="s">
         <v>29</v>
       </c>
       <c r="E10" s="5" t="s">
@@ -936,18 +961,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1249,16 +1268,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1266,5 +1291,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-07 11:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11050" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C29BEAC8-F1B8-4595-8481-9AB4F92989AC}"/>
+  <xr:revisionPtr revIDLastSave="11051" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3F39FB7-12E1-4CBF-9836-72BDBCD399F2}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -114,7 +114,7 @@
     <t>P9/S7L4-ITA</t>
   </si>
   <si>
-    <t>MRS CASTANET</t>
+    <t>MR CASTANET</t>
   </si>
   <si>
     <t>MRS MAQUET</t>
@@ -961,15 +961,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1267,6 +1258,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1283,11 +1283,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-07 16:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11051" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3F39FB7-12E1-4CBF-9836-72BDBCD399F2}"/>
+  <xr:revisionPtr revIDLastSave="11054" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{404A6044-95F0-4162-88CE-A3154828CAF9}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,116 +60,55 @@
     <t>MR ANYFANTAKIS</t>
   </si>
   <si>
-    <t>07/09</t>
-  </si>
-  <si>
-    <t>MR STEFANIS</t>
-  </si>
-  <si>
-    <t>P3/S1RORELA</t>
-  </si>
-  <si>
-    <t>A111</t>
+    <t>08/09</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
   <si>
     <t>MR HEDBERG</t>
   </si>
   <si>
-    <t>MR LEADER</t>
-  </si>
-  <si>
-    <t>P1/S7L2-ENA</t>
+    <t>MRS ZARB HABER</t>
+  </si>
+  <si>
+    <t>P4/S1L2-ENA</t>
   </si>
   <si>
     <t>C209</t>
   </si>
   <si>
-    <t>P2/S7L2-ENA</t>
-  </si>
-  <si>
-    <t>MRS WILES</t>
-  </si>
-  <si>
-    <t>P8/S4L3-ENB</t>
-  </si>
-  <si>
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
-    <t>MRS VERZELETTI</t>
-  </si>
-  <si>
-    <t>P1/S1L3-ITA</t>
+    <t>MRS ROMANO</t>
+  </si>
+  <si>
+    <t>P1/S2LATITA</t>
   </si>
   <si>
     <t>B114</t>
   </si>
   <si>
-    <t>MRS BENETTI</t>
-  </si>
-  <si>
-    <t>P5/S7L3-ITA</t>
-  </si>
-  <si>
-    <t>P9/S7L4-ITA</t>
-  </si>
-  <si>
-    <t>MR CASTANET</t>
-  </si>
-  <si>
-    <t>MRS MAQUET</t>
-  </si>
-  <si>
-    <t>P4/S2SCIFRA</t>
-  </si>
-  <si>
-    <t>D204</t>
-  </si>
-  <si>
-    <t>MRS LUC</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF000000"/>
-        <rFont val="Verdana"/>
-      </rPr>
-      <t>P7/S2SCIFR</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Verdana"/>
-      </rPr>
-      <t>D</t>
-    </r>
-  </si>
-  <si>
-    <t>D209</t>
-  </si>
-  <si>
-    <t>MRS RHEINHEIMER</t>
-  </si>
-  <si>
-    <t>P8/S2SCIFRD</t>
-  </si>
-  <si>
     <t>MRS STRAUS ZULU</t>
   </si>
   <si>
-    <t>*</t>
+    <t>MR MULRENNAN</t>
+  </si>
+  <si>
+    <t>S4/S1L2-ENE</t>
+  </si>
+  <si>
+    <t>A108</t>
   </si>
   <si>
     <t xml:space="preserve">MRS NECHITA </t>
   </si>
   <si>
-    <t>MRS CONNOLLY</t>
-  </si>
-  <si>
-    <t>P1/S1L3-ENB</t>
+    <t>MRS PATSIADOU</t>
+  </si>
+  <si>
+    <t>P4/S1L2-END</t>
   </si>
   <si>
     <t>C001</t>
@@ -178,29 +117,20 @@
     <t>MR PARKER</t>
   </si>
   <si>
-    <t>MR ATCHADE</t>
-  </si>
-  <si>
-    <t>MR NESTORAS</t>
-  </si>
-  <si>
-    <t>ONLY P2</t>
-  </si>
-  <si>
-    <t>MRS GROBER</t>
-  </si>
-  <si>
-    <t>P2/S2MATENC</t>
-  </si>
-  <si>
-    <t>B015</t>
+    <t>MR BERNET</t>
+  </si>
+  <si>
+    <t>MR O'MAHONEY</t>
+  </si>
+  <si>
+    <t>ONLY P8 TO P9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -227,30 +157,23 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FFFF0000"/>
-      <name val="Verdana"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Verdana"/>
     </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FFFF0000"/>
-      <name val="Verdana"/>
-    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -330,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -362,11 +285,8 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -691,7 +611,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U17"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -737,221 +657,122 @@
       <c r="C2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>9</v>
-      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>11</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4"/>
+      <c r="A4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C4" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C5" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
+      <c r="A7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C7" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>20</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C8" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>20</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="5" t="s">
         <v>27</v>
       </c>
+      <c r="C9" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3"/>
       <c r="B10" s="4"/>
-      <c r="C10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -961,6 +782,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1258,15 +1088,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1283,11 +1104,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-08 08:10
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11054" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{404A6044-95F0-4162-88CE-A3154828CAF9}"/>
+  <xr:revisionPtr revIDLastSave="11058" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05F85323-7C1E-4A99-BE41-46C972892F34}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
   <si>
     <t>NOMS</t>
   </si>
@@ -124,6 +124,12 @@
   </si>
   <si>
     <t>ONLY P8 TO P9</t>
+  </si>
+  <si>
+    <t>MRS VEHLING</t>
+  </si>
+  <si>
+    <t>ONLY P5</t>
   </si>
 </sst>
 </file>
@@ -611,7 +617,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -768,11 +774,38 @@
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="9"/>
+      <c r="A10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>7</v>
+      </c>
       <c r="D10" s="10"/>
       <c r="E10" s="5"/>
+    </row>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -782,15 +815,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1088,6 +1112,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1104,11 +1137,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-08 08:15
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11058" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05F85323-7C1E-4A99-BE41-46C972892F34}"/>
+  <xr:revisionPtr revIDLastSave="11063" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDF1F168-373C-482F-8E42-2E3580336DFB}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
   <si>
     <t>NOMS</t>
   </si>
@@ -130,6 +130,18 @@
   </si>
   <si>
     <t>ONLY P5</t>
+  </si>
+  <si>
+    <t>MR ATCHADE</t>
+  </si>
+  <si>
+    <t>MRS DEMARTINI</t>
+  </si>
+  <si>
+    <t>P3/S1RCADEA</t>
+  </si>
+  <si>
+    <t>B106</t>
   </si>
 </sst>
 </file>
@@ -787,11 +799,21 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="5"/>
+      <c r="A11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3"/>

</xml_diff>

<commit_message>
MAJ absences 2026-09-08 08:20
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11063" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDF1F168-373C-482F-8E42-2E3580336DFB}"/>
+  <xr:revisionPtr revIDLastSave="11068" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC201010-9B6E-4AEB-8BB7-40E63D5B359C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
   <si>
     <t>NOMS</t>
   </si>
@@ -142,6 +142,18 @@
   </si>
   <si>
     <t>B106</t>
+  </si>
+  <si>
+    <t>MR GOMPIL</t>
+  </si>
+  <si>
+    <t>ONLY P4</t>
+  </si>
+  <si>
+    <t>P4/S4RPRENA</t>
+  </si>
+  <si>
+    <t>B016</t>
   </si>
 </sst>
 </file>
@@ -816,11 +828,21 @@
       </c>
     </row>
     <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="5"/>
+      <c r="A12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="13" spans="1:12" ht="18">
       <c r="A13" s="3"/>

</xml_diff>

<commit_message>
MAJ absences 2026-09-08 09:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11068" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC201010-9B6E-4AEB-8BB7-40E63D5B359C}"/>
+  <xr:revisionPtr revIDLastSave="11073" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4D7D85F-E46C-450A-B2F6-A0FF262DBCFC}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
   <si>
     <t>NOMS</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t>ONLY P8 TO P9</t>
+  </si>
+  <si>
+    <t>MRS RASCHIATORE</t>
   </si>
   <si>
     <t>MRS VEHLING</t>
@@ -641,7 +644,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -802,54 +805,67 @@
         <v>28</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C10" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="10"/>
+      <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="C11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>33</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="D11" s="10"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:12" ht="18">
       <c r="A12" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="4" t="s">
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="B13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D12" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="5" t="s">
+      <c r="D13" s="10" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="5"/>
+      <c r="E13" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1157,15 +1173,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -1180,14 +1187,23 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-08 16:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11073" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4D7D85F-E46C-450A-B2F6-A0FF262DBCFC}"/>
+  <xr:revisionPtr revIDLastSave="11087" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2E4C608-884F-4FBE-BD52-7677A463C820}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,19 +57,13 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MR ANYFANTAKIS</t>
-  </si>
-  <si>
-    <t>08/09</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
     <t>MR HEDBERG</t>
   </si>
   <si>
-    <t>MRS ZARB HABER</t>
+    <t>09/09</t>
+  </si>
+  <si>
+    <t>MRS WILES</t>
   </si>
   <si>
     <t>P4/S1L2-ENA</t>
@@ -78,34 +72,37 @@
     <t>C209</t>
   </si>
   <si>
+    <t>MR BOTH</t>
+  </si>
+  <si>
+    <t>P8/S6PH4ENA</t>
+  </si>
+  <si>
+    <t>!A202</t>
+  </si>
+  <si>
+    <t>P9/S6PH4ENA</t>
+  </si>
+  <si>
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
     <t>MRS ROMANO</t>
   </si>
   <si>
-    <t>P1/S2LATITA</t>
+    <t>P3/S4L1-ITA</t>
   </si>
   <si>
     <t>B114</t>
   </si>
   <si>
-    <t>MRS STRAUS ZULU</t>
-  </si>
-  <si>
-    <t>MR MULRENNAN</t>
-  </si>
-  <si>
-    <t>S4/S1L2-ENE</t>
-  </si>
-  <si>
-    <t>A108</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MRS NECHITA </t>
-  </si>
-  <si>
-    <t>MRS PATSIADOU</t>
+    <t>P8/S3L1-ITB</t>
+  </si>
+  <si>
+    <t>MRS NECHITA</t>
+  </si>
+  <si>
+    <t>MRS FIORETTI</t>
   </si>
   <si>
     <t>P4/S1L2-END</t>
@@ -117,53 +114,20 @@
     <t>MR PARKER</t>
   </si>
   <si>
-    <t>MR BERNET</t>
-  </si>
-  <si>
-    <t>MR O'MAHONEY</t>
-  </si>
-  <si>
-    <t>ONLY P8 TO P9</t>
-  </si>
-  <si>
-    <t>MRS RASCHIATORE</t>
-  </si>
-  <si>
-    <t>MRS VEHLING</t>
-  </si>
-  <si>
-    <t>ONLY P5</t>
-  </si>
-  <si>
-    <t>MR ATCHADE</t>
-  </si>
-  <si>
-    <t>MRS DEMARTINI</t>
-  </si>
-  <si>
-    <t>P3/S1RCADEA</t>
-  </si>
-  <si>
-    <t>B106</t>
-  </si>
-  <si>
-    <t>MR GOMPIL</t>
-  </si>
-  <si>
-    <t>ONLY P4</t>
-  </si>
-  <si>
-    <t>P4/S4RPRENA</t>
-  </si>
-  <si>
-    <t>B016</t>
+    <t>MRS DUFF</t>
+  </si>
+  <si>
+    <t>P2/S3SCHENF</t>
+  </si>
+  <si>
+    <t>B018</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -188,11 +152,6 @@
       <color rgb="FF000000"/>
       <name val="Verdana"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Verdana"/>
     </font>
   </fonts>
   <fills count="3">
@@ -286,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -314,9 +273,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -644,7 +600,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U9"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -690,182 +646,109 @@
       <c r="C2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="D2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18.75" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>17</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="20.25" customHeight="1">
-      <c r="A6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
       <c r="C6" s="9" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+        <v>20</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="8" spans="1:12" ht="18">
       <c r="A8" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+        <v>24</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>7</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="10"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
-    </row>
-    <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C10" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D11" s="10"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -875,6 +758,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1172,32 +1079,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1205,5 +1088,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-09 08:20
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11087" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2E4C608-884F-4FBE-BD52-7677A463C820}"/>
+  <xr:revisionPtr revIDLastSave="11090" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBE90D75-B063-4646-904B-E04F05B9C03C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>NOMS</t>
   </si>
@@ -121,6 +121,12 @@
   </si>
   <si>
     <t>B018</t>
+  </si>
+  <si>
+    <t>MRS RAYMONDAUD</t>
+  </si>
+  <si>
+    <t>MRS MARTINEAU</t>
   </si>
 </sst>
 </file>
@@ -744,9 +750,15 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="10"/>
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>28</v>
+      </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
@@ -758,15 +770,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -779,6 +782,15 @@
     <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1080,11 +1092,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-09 08:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11090" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBE90D75-B063-4646-904B-E04F05B9C03C}"/>
+  <xr:revisionPtr revIDLastSave="11103" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{065C2A69-129B-4D76-B350-F2703288B22A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Feuil1!$A$1:$E$4</definedName>
     <definedName name="toShow">Feuil1!$A:$E</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
   <si>
     <t>NOMS</t>
   </si>
@@ -72,18 +72,6 @@
     <t>C209</t>
   </si>
   <si>
-    <t>MR BOTH</t>
-  </si>
-  <si>
-    <t>P8/S6PH4ENA</t>
-  </si>
-  <si>
-    <t>!A202</t>
-  </si>
-  <si>
-    <t>P9/S6PH4ENA</t>
-  </si>
-  <si>
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
@@ -127,6 +115,30 @@
   </si>
   <si>
     <t>MRS MARTINEAU</t>
+  </si>
+  <si>
+    <t>P1/S1L1-FRA</t>
+  </si>
+  <si>
+    <t>D104</t>
+  </si>
+  <si>
+    <t>MRS PIERSON</t>
+  </si>
+  <si>
+    <t>P2/S1L1-FRA</t>
+  </si>
+  <si>
+    <t>MR CHASSE</t>
+  </si>
+  <si>
+    <t>P3/S4L1-FRC</t>
+  </si>
+  <si>
+    <t>MR FABY</t>
+  </si>
+  <si>
+    <t>P8/S4L1-FRB</t>
   </si>
 </sst>
 </file>
@@ -606,7 +618,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -660,107 +672,124 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C3" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="18.75" customHeight="1">
+    <row r="4" spans="1:12" ht="20.25" customHeight="1">
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="5" t="s">
-        <v>12</v>
-      </c>
     </row>
-    <row r="5" spans="1:12" ht="18.75" customHeight="1">
+    <row r="5" spans="1:12" ht="18">
       <c r="A5" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="20.25" customHeight="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="4"/>
+    <row r="6" spans="1:12" ht="18">
+      <c r="A6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C6" s="9" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>20</v>
+      <c r="C7" s="10" t="s">
+        <v>24</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
       <c r="C8" s="9" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="18">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>26</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -770,30 +799,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1091,14 +1096,38 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-09 15:55
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11103" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{065C2A69-129B-4D76-B350-F2703288B22A}"/>
+  <xr:revisionPtr revIDLastSave="11107" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{358A8477-0191-42C4-82B8-4108AB744CCD}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
   <si>
     <t>NOMS</t>
   </si>
@@ -139,6 +139,15 @@
   </si>
   <si>
     <t>P8/S4L1-FRB</t>
+  </si>
+  <si>
+    <t>MR MORROW</t>
+  </si>
+  <si>
+    <t>ONLY P7 TO P9</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -618,7 +627,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U10"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -790,6 +799,19 @@
       <c r="E10" s="5" t="s">
         <v>26</v>
       </c>
+    </row>
+    <row r="11" spans="1:12" ht="18">
+      <c r="A11" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1097,6 +1119,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -1111,23 +1142,14 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-09 16:20
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11107" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{358A8477-0191-42C4-82B8-4108AB744CCD}"/>
+  <xr:revisionPtr revIDLastSave="11108" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88342BCB-D354-4B03-AD92-2AC23A8AB4DE}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
   <si>
     <t>NOMS</t>
   </si>
@@ -57,94 +57,85 @@
     <t>SALLES</t>
   </si>
   <si>
-    <t>MR HEDBERG</t>
+    <t>MRS PORTOGHESE</t>
   </si>
   <si>
     <t>09/09</t>
   </si>
   <si>
-    <t>MRS WILES</t>
-  </si>
-  <si>
-    <t>P4/S1L2-ENA</t>
-  </si>
-  <si>
-    <t>C209</t>
-  </si>
-  <si>
-    <t>MRS PORTOGHESE</t>
+    <t>MRS BENETTI</t>
+  </si>
+  <si>
+    <t>P4/S7L4-ITA</t>
+  </si>
+  <si>
+    <t>B114</t>
+  </si>
+  <si>
+    <t>P6/S2LATITA</t>
+  </si>
+  <si>
+    <t>MR ORIOLO</t>
+  </si>
+  <si>
+    <t>P7/S7L3-ITA</t>
   </si>
   <si>
     <t>MRS ROMANO</t>
   </si>
   <si>
-    <t>P3/S4L1-ITA</t>
-  </si>
-  <si>
-    <t>B114</t>
-  </si>
-  <si>
-    <t>P8/S3L1-ITB</t>
+    <t>P9/S4L1-ITA</t>
+  </si>
+  <si>
+    <t>MR ANYFANTAKIS</t>
+  </si>
+  <si>
+    <t>MRS ARGYRI</t>
+  </si>
+  <si>
+    <t>P4/S2RORELA</t>
+  </si>
+  <si>
+    <t>B212</t>
+  </si>
+  <si>
+    <t>MRS KASTANIDOU</t>
+  </si>
+  <si>
+    <t>P5/S3RORELA</t>
   </si>
   <si>
     <t>MRS NECHITA</t>
   </si>
   <si>
-    <t>MRS FIORETTI</t>
-  </si>
-  <si>
-    <t>P4/S1L2-END</t>
+    <t>MRS VALENTE</t>
+  </si>
+  <si>
+    <t>P1/S1L2-END</t>
   </si>
   <si>
     <t>C001</t>
   </si>
   <si>
+    <t>MR BIRCH</t>
+  </si>
+  <si>
+    <t>P2/S1L2-END</t>
+  </si>
+  <si>
     <t>MR PARKER</t>
   </si>
   <si>
-    <t>MRS DUFF</t>
-  </si>
-  <si>
-    <t>P2/S3SCHENF</t>
+    <t>MRS XEROU</t>
+  </si>
+  <si>
+    <t>P7/S3SCHENF</t>
   </si>
   <si>
     <t>B018</t>
   </si>
   <si>
-    <t>MRS RAYMONDAUD</t>
-  </si>
-  <si>
-    <t>MRS MARTINEAU</t>
-  </si>
-  <si>
-    <t>P1/S1L1-FRA</t>
-  </si>
-  <si>
-    <t>D104</t>
-  </si>
-  <si>
-    <t>MRS PIERSON</t>
-  </si>
-  <si>
-    <t>P2/S1L1-FRA</t>
-  </si>
-  <si>
-    <t>MR CHASSE</t>
-  </si>
-  <si>
-    <t>P3/S4L1-FRC</t>
-  </si>
-  <si>
-    <t>MR FABY</t>
-  </si>
-  <si>
-    <t>P8/S4L1-FRB</t>
-  </si>
-  <si>
-    <t>MR MORROW</t>
-  </si>
-  <si>
-    <t>ONLY P7 TO P9</t>
+    <t>MR ATCHADE</t>
   </si>
   <si>
     <t>*</t>
@@ -681,20 +672,16 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="18.75" customHeight="1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>12</v>
-      </c>
       <c r="E3" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="20.25" customHeight="1">
@@ -704,111 +691,111 @@
         <v>11</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18">
-      <c r="A5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="4"/>
       <c r="C5" s="9" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
       <c r="A6" s="3" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A7" s="3"/>
+      <c r="B7" s="4"/>
       <c r="C7" s="10" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C8" s="9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3"/>
       <c r="B9" s="4"/>
       <c r="C9" s="9" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3"/>
-      <c r="B10" s="4"/>
+      <c r="A10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C10" s="10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
@@ -821,6 +808,30 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1118,32 +1129,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1151,5 +1138,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-10 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11108" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88342BCB-D354-4B03-AD92-2AC23A8AB4DE}"/>
+  <xr:revisionPtr revIDLastSave="11132" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCF01CEA-B78B-47EB-9E8A-9C7EC20703EA}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,7 +60,7 @@
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
-    <t>09/09</t>
+    <t>10/09</t>
   </si>
   <si>
     <t>MRS BENETTI</t>
@@ -108,21 +108,15 @@
     <t>MRS NECHITA</t>
   </si>
   <si>
-    <t>MRS VALENTE</t>
-  </si>
-  <si>
-    <t>P1/S1L2-END</t>
+    <t>MR BIRCH</t>
+  </si>
+  <si>
+    <t>P2/S1L2-END</t>
   </si>
   <si>
     <t>C001</t>
   </si>
   <si>
-    <t>MR BIRCH</t>
-  </si>
-  <si>
-    <t>P2/S1L2-END</t>
-  </si>
-  <si>
     <t>MR PARKER</t>
   </si>
   <si>
@@ -139,6 +133,27 @@
   </si>
   <si>
     <t>*</t>
+  </si>
+  <si>
+    <t>MRS PIERSON LIENARD</t>
+  </si>
+  <si>
+    <t>MR CHASSE</t>
+  </si>
+  <si>
+    <t>P4/S2L1-FRC</t>
+  </si>
+  <si>
+    <t>C202</t>
+  </si>
+  <si>
+    <t>MRS GROBER</t>
+  </si>
+  <si>
+    <t>P5/S2LATFRA</t>
+  </si>
+  <si>
+    <t>MR MORROW</t>
   </si>
 </sst>
 </file>
@@ -618,7 +633,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -758,34 +773,34 @@
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="9" t="s">
+      <c r="A9" s="3" t="s">
         <v>25</v>
       </c>
+      <c r="B9" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>26</v>
+      </c>
       <c r="D9" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="5" t="s">
         <v>30</v>
       </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
       <c r="A11" s="3" t="s">
@@ -797,8 +812,45 @@
       <c r="C11" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="D11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -808,21 +860,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -831,7 +868,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1129,14 +1166,29 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-10 09:15
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11132" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCF01CEA-B78B-47EB-9E8A-9C7EC20703EA}"/>
+  <xr:revisionPtr revIDLastSave="11135" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF3BBCC8-B8AA-4489-9010-E06007296447}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
   <si>
     <t>NOMS</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>MR MORROW</t>
+  </si>
+  <si>
+    <t>MR WAECHTER</t>
+  </si>
+  <si>
+    <t>ONLY P2</t>
   </si>
 </sst>
 </file>
@@ -846,9 +852,15 @@
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="10"/>
+      <c r="A14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>30</v>
+      </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
     </row>
@@ -860,15 +872,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1166,6 +1169,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1182,11 +1194,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-10 10:25
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11135" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF3BBCC8-B8AA-4489-9010-E06007296447}"/>
+  <xr:revisionPtr revIDLastSave="11136" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60F552BA-EE89-4AD8-A135-C29ECE817135}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -867,11 +867,35 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1169,32 +1193,8 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1202,5 +1202,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-10 15:50
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30502"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11136" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60F552BA-EE89-4AD8-A135-C29ECE817135}"/>
+  <xr:revisionPtr revIDLastSave="11139" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2EBF39E-1FBD-4E54-83CE-F87B1624333E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,106 +60,64 @@
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
-    <t>10/09</t>
+    <t>11/09</t>
   </si>
   <si>
     <t>MRS BENETTI</t>
   </si>
   <si>
-    <t>P4/S7L4-ITA</t>
+    <t>P2/S3L1-ITB</t>
   </si>
   <si>
     <t>B114</t>
   </si>
   <si>
-    <t>P6/S2LATITA</t>
-  </si>
-  <si>
-    <t>MR ORIOLO</t>
-  </si>
-  <si>
-    <t>P7/S7L3-ITA</t>
+    <t>MRS GIORGERINI</t>
+  </si>
+  <si>
+    <t>P5/S7L4-ITA</t>
+  </si>
+  <si>
+    <t>P7/S1L3-ITA</t>
   </si>
   <si>
     <t>MRS ROMANO</t>
   </si>
   <si>
-    <t>P9/S4L1-ITA</t>
-  </si>
-  <si>
-    <t>MR ANYFANTAKIS</t>
-  </si>
-  <si>
-    <t>MRS ARGYRI</t>
-  </si>
-  <si>
-    <t>P4/S2RORELA</t>
-  </si>
-  <si>
-    <t>B212</t>
-  </si>
-  <si>
-    <t>MRS KASTANIDOU</t>
-  </si>
-  <si>
-    <t>P5/S3RORELA</t>
+    <t>P8/S4L1-ITA</t>
+  </si>
+  <si>
+    <t>P9/S3LATITA</t>
   </si>
   <si>
     <t>MRS NECHITA</t>
   </si>
   <si>
-    <t>MR BIRCH</t>
-  </si>
-  <si>
-    <t>P2/S1L2-END</t>
+    <t>MR MARTINEK</t>
+  </si>
+  <si>
+    <t>P6/S1L2-END</t>
   </si>
   <si>
     <t>C001</t>
   </si>
   <si>
+    <t>MRS JUHASZ</t>
+  </si>
+  <si>
+    <t>P7/S1L3-ENB</t>
+  </si>
+  <si>
     <t>MR PARKER</t>
   </si>
   <si>
-    <t>MRS XEROU</t>
-  </si>
-  <si>
-    <t>P7/S3SCHENF</t>
-  </si>
-  <si>
-    <t>B018</t>
-  </si>
-  <si>
-    <t>MR ATCHADE</t>
-  </si>
-  <si>
     <t>*</t>
   </si>
   <si>
-    <t>MRS PIERSON LIENARD</t>
-  </si>
-  <si>
-    <t>MR CHASSE</t>
-  </si>
-  <si>
-    <t>P4/S2L1-FRC</t>
-  </si>
-  <si>
-    <t>C202</t>
-  </si>
-  <si>
-    <t>MRS GROBER</t>
-  </si>
-  <si>
-    <t>P5/S2LATFRA</t>
-  </si>
-  <si>
-    <t>MR MORROW</t>
-  </si>
-  <si>
-    <t>MR WAECHTER</t>
-  </si>
-  <si>
-    <t>ONLY P2</t>
+    <t>MRS MORAWSKA</t>
+  </si>
+  <si>
+    <t>ONLY P3 TO P4</t>
   </si>
 </sst>
 </file>
@@ -639,7 +597,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -696,10 +654,10 @@
       <c r="A3" s="3"/>
       <c r="B3" s="4"/>
       <c r="C3" s="9" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>9</v>
@@ -709,7 +667,7 @@
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>12</v>
@@ -732,137 +690,80 @@
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>17</v>
-      </c>
       <c r="E6" s="5" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="10" t="s">
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="E8" s="5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
       <c r="A9" s="3" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>28</v>
-      </c>
+      <c r="C9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:12" ht="18">
       <c r="A10" s="3" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -872,6 +773,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -884,15 +794,6 @@
     <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1194,11 +1095,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-11 08:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11139" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2EBF39E-1FBD-4E54-83CE-F87B1624333E}"/>
+  <xr:revisionPtr revIDLastSave="11146" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75D49286-FCD7-4C97-ADAA-2EB31D5892D7}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
   <si>
     <t>NOMS</t>
   </si>
@@ -118,6 +118,12 @@
   </si>
   <si>
     <t>ONLY P3 TO P4</t>
+  </si>
+  <si>
+    <t>MRS FERRARI</t>
+  </si>
+  <si>
+    <t>MR MORROW</t>
   </si>
 </sst>
 </file>
@@ -597,7 +603,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U14"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -759,11 +765,44 @@
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="10"/>
+      <c r="A11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>23</v>
+      </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
+    </row>
+    <row r="12" spans="1:12" ht="18">
+      <c r="A12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+    </row>
+    <row r="13" spans="1:12" ht="18">
+      <c r="A13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+    </row>
+    <row r="14" spans="1:12" ht="18">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -773,30 +812,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1094,8 +1109,32 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1103,5 +1142,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-11 08:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11146" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75D49286-FCD7-4C97-ADAA-2EB31D5892D7}"/>
+  <xr:revisionPtr revIDLastSave="11161" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0AE504A-89FE-4764-89EA-84F52722A5A8}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="36">
   <si>
     <t>NOMS</t>
   </si>
@@ -124,6 +124,30 @@
   </si>
   <si>
     <t>MR MORROW</t>
+  </si>
+  <si>
+    <t>MRS PIERSON LIENARD</t>
+  </si>
+  <si>
+    <t>MRS GARCIA PILAR</t>
+  </si>
+  <si>
+    <t>P3/S2MORFRA</t>
+  </si>
+  <si>
+    <t>C202</t>
+  </si>
+  <si>
+    <t>MR GLASNOVIC</t>
+  </si>
+  <si>
+    <t>P4/S2LATFRA</t>
+  </si>
+  <si>
+    <t>MRS DESROSIERS</t>
+  </si>
+  <si>
+    <t>P8/S2L1-FRC</t>
   </si>
 </sst>
 </file>
@@ -603,7 +627,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:U15"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -791,18 +815,47 @@
       <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="A13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="14" spans="1:12" ht="18">
       <c r="A14" s="3"/>
       <c r="B14" s="4"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="C14" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18">
+      <c r="A15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>31</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
MAJ absences 2026-09-11 08:15
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11161" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0AE504A-89FE-4764-89EA-84F52722A5A8}"/>
+  <xr:revisionPtr revIDLastSave="11168" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E11E9E02-7A39-4059-8E96-89022D85FC3B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="40">
   <si>
     <t>NOMS</t>
   </si>
@@ -148,6 +148,18 @@
   </si>
   <si>
     <t>P8/S2L1-FRC</t>
+  </si>
+  <si>
+    <t>MR ATCHADE</t>
+  </si>
+  <si>
+    <t>MRS TOURA</t>
+  </si>
+  <si>
+    <t>P3/S2RCADEA</t>
+  </si>
+  <si>
+    <t>B010</t>
   </si>
 </sst>
 </file>
@@ -627,7 +639,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -855,6 +867,23 @@
       </c>
       <c r="E15" s="5" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="18">
+      <c r="A16" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MAJ absences 2026-09-11 08:30
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11168" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E11E9E02-7A39-4059-8E96-89022D85FC3B}"/>
+  <xr:revisionPtr revIDLastSave="11169" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0BC6A8E-7B1B-4F4D-993F-F2217C6E584A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -93,7 +93,7 @@
     <t>MRS NECHITA</t>
   </si>
   <si>
-    <t>MR MARTINEK</t>
+    <t>MRS GARAFOL</t>
   </si>
   <si>
     <t>P6/S1L2-END</t>

</xml_diff>

<commit_message>
MAJ absences 2026-09-11 10:00
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11169" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0BC6A8E-7B1B-4F4D-993F-F2217C6E584A}"/>
+  <xr:revisionPtr revIDLastSave="11183" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B09E6940-D129-432F-8B47-330FCDA9800A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
   <si>
     <t>NOMS</t>
   </si>
@@ -160,6 +160,21 @@
   </si>
   <si>
     <t>B010</t>
+  </si>
+  <si>
+    <t>!Mr HEDBERG</t>
+  </si>
+  <si>
+    <t>!ONLY P7</t>
+  </si>
+  <si>
+    <t>!MR SAMMUT</t>
+  </si>
+  <si>
+    <t>!P7/S7L2-ENA</t>
+  </si>
+  <si>
+    <t>!C209</t>
   </si>
 </sst>
 </file>
@@ -639,7 +654,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U16"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -885,6 +900,30 @@
       <c r="E16" s="5" t="s">
         <v>39</v>
       </c>
+    </row>
+    <row r="17" spans="1:5" ht="18">
+      <c r="A17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1192,6 +1231,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
@@ -1206,23 +1254,14 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>

<commit_message>
MAJ absences 2026-09-11 10:05
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11183" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B09E6940-D129-432F-8B47-330FCDA9800A}"/>
+  <xr:revisionPtr revIDLastSave="11185" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02A6DFA6-929C-4412-BFEB-24C8551138A5}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -162,7 +162,7 @@
     <t>B010</t>
   </si>
   <si>
-    <t>!Mr HEDBERG</t>
+    <t>MR HEDBERG</t>
   </si>
   <si>
     <t>!ONLY P7</t>
@@ -933,6 +933,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1230,15 +1239,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1255,11 +1255,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
MAJ absences 2026-09-11 16:35
</commit_message>
<xml_diff>
--- a/Absences_Sharepoint.xlsx
+++ b/Absences_Sharepoint.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eursc-my.sharepoint.com/personal/mathiere_eursc_eu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11185" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02A6DFA6-929C-4412-BFEB-24C8551138A5}"/>
+  <xr:revisionPtr revIDLastSave="11189" documentId="13_ncr:1_{D8C8AC21-DC92-474D-84DE-8D29D0988F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{726F75C0-755A-40C3-AE7F-693244006EA4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3740289B-832A-4290-BDF4-CA7ADE3B0EEE}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
   <si>
     <t>NOMS</t>
   </si>
@@ -60,121 +60,73 @@
     <t>MRS PORTOGHESE</t>
   </si>
   <si>
-    <t>11/09</t>
+    <t>14/09</t>
+  </si>
+  <si>
+    <t>MRS VERZELETTI</t>
+  </si>
+  <si>
+    <t>P1/S1L3ITA</t>
+  </si>
+  <si>
+    <t>B114</t>
   </si>
   <si>
     <t>MRS BENETTI</t>
   </si>
   <si>
-    <t>P2/S3L1-ITB</t>
-  </si>
-  <si>
-    <t>B114</t>
-  </si>
-  <si>
-    <t>MRS GIORGERINI</t>
-  </si>
-  <si>
-    <t>P5/S7L4-ITA</t>
-  </si>
-  <si>
-    <t>P7/S1L3-ITA</t>
-  </si>
-  <si>
-    <t>MRS ROMANO</t>
-  </si>
-  <si>
-    <t>P8/S4L1-ITA</t>
-  </si>
-  <si>
-    <t>P9/S3LATITA</t>
-  </si>
-  <si>
-    <t>MRS NECHITA</t>
-  </si>
-  <si>
-    <t>MRS GARAFOL</t>
-  </si>
-  <si>
-    <t>P6/S1L2-END</t>
-  </si>
-  <si>
-    <t>C001</t>
-  </si>
-  <si>
-    <t>MRS JUHASZ</t>
-  </si>
-  <si>
-    <t>P7/S1L3-ENB</t>
-  </si>
-  <si>
-    <t>MR PARKER</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>MRS MORAWSKA</t>
-  </si>
-  <si>
-    <t>ONLY P3 TO P4</t>
-  </si>
-  <si>
-    <t>MRS FERRARI</t>
-  </si>
-  <si>
-    <t>MR MORROW</t>
-  </si>
-  <si>
-    <t>MRS PIERSON LIENARD</t>
-  </si>
-  <si>
-    <t>MRS GARCIA PILAR</t>
-  </si>
-  <si>
-    <t>P3/S2MORFRA</t>
-  </si>
-  <si>
-    <t>C202</t>
-  </si>
-  <si>
-    <t>MR GLASNOVIC</t>
-  </si>
-  <si>
-    <t>P4/S2LATFRA</t>
-  </si>
-  <si>
-    <t>MRS DESROSIERS</t>
-  </si>
-  <si>
-    <t>P8/S2L1-FRC</t>
-  </si>
-  <si>
-    <t>MR ATCHADE</t>
-  </si>
-  <si>
-    <t>MRS TOURA</t>
-  </si>
-  <si>
-    <t>P3/S2RCADEA</t>
-  </si>
-  <si>
-    <t>B010</t>
+    <t>P5/S7L3-ITA</t>
+  </si>
+  <si>
+    <t>P9/S7L4-ITA</t>
   </si>
   <si>
     <t>MR HEDBERG</t>
   </si>
   <si>
-    <t>!ONLY P7</t>
-  </si>
-  <si>
-    <t>!MR SAMMUT</t>
-  </si>
-  <si>
-    <t>!P7/S7L2-ENA</t>
-  </si>
-  <si>
-    <t>!C209</t>
+    <t>ONLY P1 TO P2</t>
+  </si>
+  <si>
+    <t>MR LEADER</t>
+  </si>
+  <si>
+    <t>P1/S7L2-ENA</t>
+  </si>
+  <si>
+    <t>C209</t>
+  </si>
+  <si>
+    <t>P2/S7L2-ENA</t>
+  </si>
+  <si>
+    <t>MRS PINHEIRO</t>
+  </si>
+  <si>
+    <t>MR NIKITOPOULOS</t>
+  </si>
+  <si>
+    <t>P5/S2EP--J</t>
+  </si>
+  <si>
+    <t>MR ANYFANTAKIS</t>
+  </si>
+  <si>
+    <t>MRS  FRYGANA</t>
+  </si>
+  <si>
+    <t>P2/S3RORELA</t>
+  </si>
+  <si>
+    <t>A111</t>
+  </si>
+  <si>
+    <t>MR KARAGIANNIS</t>
+  </si>
+  <si>
+    <t>P3/S1RORELA</t>
+  </si>
+  <si>
+    <t>P4/S2RORELA</t>
   </si>
 </sst>
 </file>
@@ -654,7 +606,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:U18"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.5703125" customWidth="1"/>
@@ -724,7 +676,7 @@
       <c r="A4" s="3"/>
       <c r="B4" s="4"/>
       <c r="C4" s="9" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>12</v>
@@ -734,196 +686,99 @@
       </c>
     </row>
     <row r="5" spans="1:12" ht="18">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="C5" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="18">
       <c r="A6" s="3"/>
       <c r="B6" s="4"/>
       <c r="C6" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="18">
       <c r="A7" s="3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>19</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:12" ht="18">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="C8" s="9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="18">
-      <c r="A9" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="4"/>
       <c r="C9" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+        <v>26</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="10" spans="1:12" ht="18">
-      <c r="A10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:12" ht="18">
-      <c r="A11" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>23</v>
-      </c>
+      <c r="A11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="10"/>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:12" ht="18">
-      <c r="A12" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" ht="18">
-      <c r="A13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="18">
-      <c r="A14" s="3"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="18">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="18">
-      <c r="A16" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="18">
-      <c r="A17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="18">
-      <c r="A18" s="3"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -933,6 +788,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
+    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -941,7 +811,7 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100072688EA0209CC47858AAB8945FA31A2" ma:contentTypeVersion="29" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b4a100729e7cd6a73b1022839a03701c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34275c52-51ce-4086-b958-e6c40ec3ced6" xmlns:ns3="4ed1dcf9-06b3-4a91-867a-d1f749225c61" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f1aabc9b86d97c8b43b23ba4e5c47e5" ns2:_="" ns3:_="">
     <xsd:import namespace="34275c52-51ce-4086-b958-e6c40ec3ced6"/>
@@ -1239,29 +1109,14 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Langages xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <TaxCatchAll xmlns="4ed1dcf9-06b3-4a91-867a-d1f749225c61" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <Service xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-    <Category xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6">Administration</Category>
-    <Images xmlns="34275c52-51ce-4086-b958-e6c40ec3ced6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76567078-8820-4013-8007-6362595EECB8}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F749EAC-3375-4A33-B2F4-3B98563F427C}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F947B5AE-3530-42B1-89EC-923DC2A63D62}"/>
 </file>
</xml_diff>